<commit_message>
Auto: parallel discovery branch 11 own-file progress (반복 3, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_11.xlsx
+++ b/output/discovery_result_11.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$A$1</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$16</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A1"/>
+  <dimension ref="A1:J16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -445,10 +445,674 @@
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="n"/>
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>큐텐상품번호</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>상점ID</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>상품명(원본)</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>한글검증명칭</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>브랜드</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>가격(엔)</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>리뷰수</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>옵션있음</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>카테고리코드</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>상품URL</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" t="inlineStr">
+        <is>
+          <t>1213065508</t>
+        </is>
+      </c>
+      <c r="B2" t="inlineStr">
+        <is>
+          <t>deesse1128</t>
+        </is>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>【2026新作】ダルバ エアフィット ブルー トーンアップUVパウダー 5.5g SPF UVケア 毛穴カバー テカリケア ヴィーガン</t>
+        </is>
+      </c>
+      <c r="E2" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F2" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G2" t="n">
+        <v>0</v>
+      </c>
+      <c r="H2" t="b">
+        <v>0</v>
+      </c>
+      <c r="I2" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213065508</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>1184719855</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>deesse1128</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>[新作]ローズマリー PDRN クーリング 脱毛シャンプー 400ml #EGF 頭皮鎮静 脱毛ケア/ローズマリー PDRN クールスカルプシャンプー/根元からふんわりボリュームケア</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G3" t="n">
+        <v>0</v>
+      </c>
+      <c r="H3" t="b">
+        <v>0</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1184719855</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>1211478917</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>deesse1128</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>【26年新リニューアル】ダルバ ヴィーガン ヘアパフュームセラム 100ml ヘアミスト 保湿 ダメージケア 韓国コスメプロフェッショナルリペアリングヘアパフュームセラム</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>3100</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0</v>
+      </c>
+      <c r="H4" t="b">
+        <v>0</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211478917</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>1211980957</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>deesse1128</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>【NEW】オウズナリー ビタ3 オーロラミスト 60ml メイクキープ ツヤミスト 保湿 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>オーズナリー</t>
+        </is>
+      </c>
+      <c r="F5" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H5" t="b">
+        <v>0</v>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211980957</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>1178226810</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>rarimarket</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>[NEW]PDRNピンクコラーゲンボリュームマルチバーム 10g/PDRN Pink Collagen Volume Multi Balm</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F6" t="n">
+        <v>4190</v>
+      </c>
+      <c r="G6" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" t="b">
+        <v>0</v>
+      </c>
+      <c r="I6" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178226810</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>1178226702</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>rarimarket</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>[1+1]ティーツリーシカポア鼻パック 5枚</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F7" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G7" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" t="b">
+        <v>0</v>
+      </c>
+      <c r="I7" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178226702</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>1178226617</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>rarimarket</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>オールデイ メイクアップ フィクサー 75ml/SO.NATURAL/FIXX/ALL DAY/MAKE UP SETTING</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>ソーナチュラル</t>
+        </is>
+      </c>
+      <c r="F8" t="n">
+        <v>1999</v>
+      </c>
+      <c r="G8" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" t="b">
+        <v>0</v>
+      </c>
+      <c r="I8" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1178226617</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>1206008325</t>
+        </is>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>DreamWish</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>ペプチドショット2X 弾力アンプル 30ml（ハリ感ケア／保湿／弾力サポート美容液）</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>アンプルエヌ</t>
+        </is>
+      </c>
+      <c r="F9" t="n">
+        <v>2122</v>
+      </c>
+      <c r="G9" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" t="b">
+        <v>0</v>
+      </c>
+      <c r="I9" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J9" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206008325</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>1206008294</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>DreamWish</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>ウォーターフィット リカバー BBクリーム 30ml #SPF40 PA+++ #保湿密着</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>セルフュージョンC</t>
+        </is>
+      </c>
+      <c r="F10" t="n">
+        <v>2927</v>
+      </c>
+      <c r="G10" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" t="b">
+        <v>0</v>
+      </c>
+      <c r="I10" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J10" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206008294</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>1174866024</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>247GOODLUCK</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>グレーズ ヘアパフュームオイル 45ml</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>ケラスターゼ</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>7405</v>
+      </c>
+      <c r="G11" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" t="b">
+        <v>0</v>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174866024</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>1206005784</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>busanjin</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>ローズオブセッション ティント 24種（グロウ/マット）</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>フィー</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>1897</v>
+      </c>
+      <c r="G12" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" t="b">
+        <v>0</v>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206005784</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>1162170897</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>berrymuch</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>[25SS/New] PDRN ヒアルロン酸 カプセル100 セラムマスク 10枚入</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>2640</v>
+      </c>
+      <c r="G13" t="n">
+        <v>7</v>
+      </c>
+      <c r="H13" t="b">
+        <v>0</v>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162170897</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>1205905275</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>berrymuch</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>アトバリア365 カプセルトナー 300ml #高密度セラミドカプセル #PHA #弱酸性 #26年5月発売</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>3531</v>
+      </c>
+      <c r="G14" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" t="b">
+        <v>0</v>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205905275</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>1204558349</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>siriya</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>リポソームバブルブースター 95ml 2種（コラーゲン／キャビア PDRN）から1つ選択</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F15" t="n">
+        <v>3498</v>
+      </c>
+      <c r="G15" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" t="b">
+        <v>0</v>
+      </c>
+      <c r="I15" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204558349</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>1203110839</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>siriya</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>イレイザー ショット グリコリック酸ブースター 30ml #皮脂・角質除去</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>アレンシア</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>4038</v>
+      </c>
+      <c r="G16" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" t="b">
+        <v>0</v>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203110839</t>
+        </is>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:A1"/>
+  <autoFilter ref="A1:J16"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 11 own-file progress (반복 6, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_11.xlsx
+++ b/output/discovery_result_11.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$16</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$38</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J16"/>
+  <dimension ref="A1:J38"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -1111,8 +1111,910 @@
         </is>
       </c>
     </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>1136214702</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>JUNSTAR</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>[シミ/白玉セット] グルタチオングロウアンプル 30ml + ディープ ビタC カプセル クリーム 55ml</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>5990</v>
+      </c>
+      <c r="G17" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" t="b">
+        <v>0</v>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1136214702</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>1190200956</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>JUNSTAR</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>クリムゾン スカイ(ポリッシュ) 8ml #シャンパンスパークル #イブニングパーティー</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>FINGER SUIT</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>2624</v>
+      </c>
+      <c r="G18" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" t="b">
+        <v>0</v>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190200956</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>1194311832</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>JUNSTAR</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>レッド イレイジングクリーム 2.0 (リニューアル) 50ml</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>2490</v>
+      </c>
+      <c r="G19" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" t="b">
+        <v>0</v>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194311832</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>1188287748</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>JUNSTAR</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>[大容量]ダーマソルトクリーム120ml</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>ABpharm</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>10990</v>
+      </c>
+      <c r="G20" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" t="b">
+        <v>0</v>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188287748</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>1176547134</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>JUNSTAR</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>ポメロ(ポリッシュ) 8ml #シナモンラテ #ピーチオレンジグリッター</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>FINGER SUIT</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>2090</v>
+      </c>
+      <c r="G21" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" t="b">
+        <v>0</v>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176547134</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>1209979406</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>onnicosme</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>【正規品】ハンーユル 幼いヨモギ 皮脂吸着 ヨモギ餅パックフォーム 120ml, 1個</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>ハンユル</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>3450</v>
+      </c>
+      <c r="G22" t="n">
+        <v>1</v>
+      </c>
+      <c r="H22" t="b">
+        <v>0</v>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209979406</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>1204386062</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>onnicosme</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>【正規品】朝鮮の美女 人参アイクリーム 30ml（ビタミンA レチナール リポソーム）</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>2890</v>
+      </c>
+      <c r="G23" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" t="b">
+        <v>0</v>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204386062</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>1203715344</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>onnicosme</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>【正規品】 フォア パーフェクティング コラーゲン ペプチド クリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Biodance</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>4190</v>
+      </c>
+      <c r="G24" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" t="b">
+        <v>0</v>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203715344</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>1202714464</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>onnicosme</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>【正規品】 マデカーメラキャプチャーアンプルパッド60枚x2個</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>3890</v>
+      </c>
+      <c r="G25" t="n">
+        <v>1</v>
+      </c>
+      <c r="H25" t="b">
+        <v>0</v>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202714464</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>1200863342</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>DEdge</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>[テミンのフォトカード100%プレゼント] マスターズ アイシー ジェリー サンスティック 14g</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>AHC</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>3459</v>
+      </c>
+      <c r="G26" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" t="b">
+        <v>0</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200863342</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>1209710276</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>DEdge</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>[26SS/New]パフュームヘアシャンプー 530ml（+100ml） #Angel muguet発売</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>La'dor</t>
+        </is>
+      </c>
+      <c r="F27" t="n">
+        <v>4344</v>
+      </c>
+      <c r="G27" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" t="b">
+        <v>0</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209710276</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>1202412626</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>DEdge</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>パーフェクトフレッシュ メンズ 男性用洗浄剤 150ml</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>ベントン</t>
+        </is>
+      </c>
+      <c r="F28" t="n">
+        <v>4000</v>
+      </c>
+      <c r="G28" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" t="b">
+        <v>0</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202412626</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>1196939883</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>DEdge</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>レチナール アイセラム リフティングローラー 15ml #カフェイン #バクチオール #アンチエイジングアプリケーター</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>アビブ</t>
+        </is>
+      </c>
+      <c r="F29" t="n">
+        <v>5063</v>
+      </c>
+      <c r="G29" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" t="b">
+        <v>0</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196939883</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>1146350889</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>seoulselectstore</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>トコフェロールビタミンEオイル原液10ml×6本 高濃度美容オイル 保湿ケア 大容量お得セット</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>マルグルダム</t>
+        </is>
+      </c>
+      <c r="F30" t="n">
+        <v>5870</v>
+      </c>
+      <c r="G30" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" t="b">
+        <v>0</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1146350889</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>1134579258</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>seoulselectstore</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>【New】グロウターンエクソソームデュアルラッシュセラム まつ毛美容液 眉毛 育毛 韓国コスメ 24時間ケア エクソソーム 二重 まつ毛ケア 長くなる</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>lily eve</t>
+        </is>
+      </c>
+      <c r="F31" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G31" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" t="b">
+        <v>0</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1134579258</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>1135156427</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>allkbeauty</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>[ブラックヘッドクレンジングセット]ゼロポアブラックヘッドディープクレンジングオイル 205ml+ゼロフォームクレンザー 120g+ブラックヘッド毛穴ブラシプレゼン/zero pore</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F32" t="n">
+        <v>3990</v>
+      </c>
+      <c r="G32" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" t="b">
+        <v>0</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1135156427</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>1193966544</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>jandb</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>Celladix トリプルレチノールウォッシュピール 30ml/Triple Retinol Wash Peel/3x</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>セラディックス</t>
+        </is>
+      </c>
+      <c r="F33" t="n">
+        <v>4900</v>
+      </c>
+      <c r="G33" t="n">
+        <v>2</v>
+      </c>
+      <c r="H33" t="b">
+        <v>0</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193966544</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>1116658196</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>jandb</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>PDRN ピーディーアールエヌ ヒアルロン酸カプセル 100セラム 30ml+リフィル30ml</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F34" t="n">
+        <v>3990</v>
+      </c>
+      <c r="G34" t="n">
+        <v>2</v>
+      </c>
+      <c r="H34" t="b">
+        <v>0</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J34" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1116658196</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>1104859818</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>jandb</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>[ビタ3種セット] ビタミストセラム8％70ml＋ビタトーニングカプセルセラム100ml＋ビタトーニングセラムローション100ml／カプセルクリーム55g</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F35" t="n">
+        <v>9190</v>
+      </c>
+      <c r="G35" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" t="b">
+        <v>0</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J35" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1104859818</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>1210644526</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>trailblue2</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>[26SS/New]レチナルペプチドセラム 30ml #ナノレチナール #ボツリヌスペプチド #9種ペプチド</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F36" t="n">
+        <v>4190</v>
+      </c>
+      <c r="G36" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" t="b">
+        <v>0</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J36" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210644526</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>1203041226</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>trailblue2</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>(ポケモンエディション)体臭ソリューション デオドラント ボディウォッシュ 720ml 2種から1つ選択</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>46CM</t>
+        </is>
+      </c>
+      <c r="F37" t="n">
+        <v>2490</v>
+      </c>
+      <c r="G37" t="n">
+        <v>0</v>
+      </c>
+      <c r="H37" t="b">
+        <v>0</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J37" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203041226</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>1187774792</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>trailblue2</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>[25SS/新作](+セボムミスト贈呈)フレッシュセボム ヘアマスカラ</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>narka</t>
+        </is>
+      </c>
+      <c r="F38" t="n">
+        <v>2249</v>
+      </c>
+      <c r="G38" t="n">
+        <v>0</v>
+      </c>
+      <c r="H38" t="b">
+        <v>0</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J38" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1187774792</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J16"/>
+  <autoFilter ref="A1:J38"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 11 own-file progress (반복 9, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_11.xlsx
+++ b/output/discovery_result_11.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$73</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J54"/>
+  <dimension ref="A1:J73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2669,8 +2669,787 @@
         </is>
       </c>
     </row>
+    <row r="55">
+      <c r="A55" t="inlineStr">
+        <is>
+          <t>1122759019</t>
+        </is>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>leekorea</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>【大容量】リフィル/本品/クリームスキン ローション 化粧水 ローション しっとり さっぱり うるおい 乾燥肌 混合肌 オイリー肌 韓国 韓国コスメ アモーレパシフィック</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>ラネージュ</t>
+        </is>
+      </c>
+      <c r="F55" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G55" t="n">
+        <v>3</v>
+      </c>
+      <c r="H55" t="b">
+        <v>0</v>
+      </c>
+      <c r="I55" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1122759019</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>1199397191</t>
+        </is>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>glovey</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>マスクフィット メイクキープ ミスト 密着キープ 崩れ防止 レッド 80ml</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>ティルティル</t>
+        </is>
+      </c>
+      <c r="F56" t="n">
+        <v>2250</v>
+      </c>
+      <c r="G56" t="n">
+        <v>5</v>
+      </c>
+      <c r="H56" t="b">
+        <v>0</v>
+      </c>
+      <c r="I56" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199397191</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>1198611443</t>
+        </is>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>glovey</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>マダガスカルセンテラアンプル 100ml</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F57" t="n">
+        <v>3130</v>
+      </c>
+      <c r="G57" t="n">
+        <v>1</v>
+      </c>
+      <c r="H57" t="b">
+        <v>0</v>
+      </c>
+      <c r="I57" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198611443</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
+        <is>
+          <t>1197582691</t>
+        </is>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>glovey</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>ナイアシンアミド 10 トラネキサミック酸 4 ダークスポット コレクティング セラム 30ml</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>アヌア</t>
+        </is>
+      </c>
+      <c r="F58" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G58" t="n">
+        <v>4</v>
+      </c>
+      <c r="H58" t="b">
+        <v>0</v>
+      </c>
+      <c r="I58" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1197582691</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="inlineStr">
+        <is>
+          <t>1208272698</t>
+        </is>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>glovey</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>レッドイレイジングクリーム 2.0 50ml</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F59" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G59" t="n">
+        <v>0</v>
+      </c>
+      <c r="H59" t="b">
+        <v>0</v>
+      </c>
+      <c r="I59" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208272698</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="inlineStr">
+        <is>
+          <t>1208271013</t>
+        </is>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>glovey</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>コラーゲンジェリークリーム 110ml</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F60" t="n">
+        <v>3930</v>
+      </c>
+      <c r="G60" t="n">
+        <v>0</v>
+      </c>
+      <c r="H60" t="b">
+        <v>0</v>
+      </c>
+      <c r="I60" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208271013</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="inlineStr">
+        <is>
+          <t>1209088264</t>
+        </is>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>GloryofSeoul</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>Centella Poremizing Clear Ampoule Pad , 60 Pads</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F61" t="n">
+        <v>2112</v>
+      </c>
+      <c r="G61" t="n">
+        <v>0</v>
+      </c>
+      <c r="H61" t="b">
+        <v>0</v>
+      </c>
+      <c r="I61" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209088264</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="inlineStr">
+        <is>
+          <t>1190423964</t>
+        </is>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>GloryofSeoul</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>Pore+Dark Spot Brightening Cream 35ml</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F62" t="n">
+        <v>1980</v>
+      </c>
+      <c r="G62" t="n">
+        <v>4</v>
+      </c>
+      <c r="H62" t="b">
+        <v>0</v>
+      </c>
+      <c r="I62" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J62" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1190423964</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="inlineStr">
+        <is>
+          <t>1094393233</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>GYUWOO</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>THEビタAレチナールショットタイトニングブースター 15ml</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F63" t="n">
+        <v>1650</v>
+      </c>
+      <c r="G63" t="n">
+        <v>4</v>
+      </c>
+      <c r="H63" t="b">
+        <v>0</v>
+      </c>
+      <c r="I63" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1094393233</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
+          <t>1119604228</t>
+        </is>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>GYUWOO</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>シカ消しゴムパッド 60枚</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F64" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G64" t="n">
+        <v>3</v>
+      </c>
+      <c r="H64" t="b">
+        <v>0</v>
+      </c>
+      <c r="I64" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J64" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1119604228</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="inlineStr">
+        <is>
+          <t>1119598747</t>
+        </is>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>GYUWOO</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>ノニアクネバブルクレンザー 155ml</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>celimax</t>
+        </is>
+      </c>
+      <c r="F65" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G65" t="n">
+        <v>1</v>
+      </c>
+      <c r="H65" t="b">
+        <v>0</v>
+      </c>
+      <c r="I65" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J65" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1119598747</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="inlineStr">
+        <is>
+          <t>1183043654</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>PICNICKOREA</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>1025独島クレンザー 弱酸性 洗顔フォーム 海洋深層水 ミネラル配合 150ml</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>ROUND LAB</t>
+        </is>
+      </c>
+      <c r="F66" t="n">
+        <v>1890</v>
+      </c>
+      <c r="G66" t="n">
+        <v>2</v>
+      </c>
+      <c r="H66" t="b">
+        <v>0</v>
+      </c>
+      <c r="I66" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J66" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183043654</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>1077111817</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>PICNICKOREA</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>オリジナル カタツムリ マスクパック 10枚セット / 保湿 弾力 潤い 肌荒れ ケア スキンケア 毎日パック 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>ジャミンギョン</t>
+        </is>
+      </c>
+      <c r="F67" t="n">
+        <v>1890</v>
+      </c>
+      <c r="G67" t="n">
+        <v>1</v>
+      </c>
+      <c r="H67" t="b">
+        <v>0</v>
+      </c>
+      <c r="I67" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J67" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1077111817</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
+          <t>1210090249</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>PICNICKOREA</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>ビタミンCブースターショット 1+1セット フェイス&amp;amp;アイクリーム くすみ・色素沈着ケア グルタチオン配合 30ml×2本</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>アレンシア</t>
+        </is>
+      </c>
+      <c r="F68" t="n">
+        <v>3150</v>
+      </c>
+      <c r="G68" t="n">
+        <v>0</v>
+      </c>
+      <c r="H68" t="b">
+        <v>0</v>
+      </c>
+      <c r="I68" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J68" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210090249</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>1173421783</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>MEWA</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>プロ ダメージヘア ヘアブラシ （4種選択1）</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>タングルエンジェル</t>
+        </is>
+      </c>
+      <c r="F69" t="n">
+        <v>2990</v>
+      </c>
+      <c r="G69" t="n">
+        <v>1</v>
+      </c>
+      <c r="H69" t="b">
+        <v>0</v>
+      </c>
+      <c r="I69" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J69" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1173421783</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>1165210718</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>MEWA</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>レチノール 1% スクアランセラム 30ml</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>ジオーディナリー</t>
+        </is>
+      </c>
+      <c r="F70" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G70" t="n">
+        <v>1</v>
+      </c>
+      <c r="H70" t="b">
+        <v>0</v>
+      </c>
+      <c r="I70" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J70" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1165210718</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
+          <t>1198551506</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>nekohime</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>ムード ペブル ハードナー (コーティングミルク/ピーチガード/ナッティコア/ベリーバリア)</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>ロムアンド</t>
+        </is>
+      </c>
+      <c r="F71" t="n">
+        <v>1512</v>
+      </c>
+      <c r="G71" t="n">
+        <v>0</v>
+      </c>
+      <c r="H71" t="b">
+        <v>0</v>
+      </c>
+      <c r="I71" t="inlineStr">
+        <is>
+          <t>120000021</t>
+        </is>
+      </c>
+      <c r="J71" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198551506</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>1161381618</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>nekohime</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>サンマデカクリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F72" t="n">
+        <v>1654</v>
+      </c>
+      <c r="G72" t="n">
+        <v>0</v>
+      </c>
+      <c r="H72" t="b">
+        <v>0</v>
+      </c>
+      <c r="I72" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J72" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1161381618</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
+          <t>1204176921</t>
+        </is>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>nekohime</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>[medicube] ブラックヘッド毛穴ブラシ</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F73" t="n">
+        <v>1690</v>
+      </c>
+      <c r="G73" t="n">
+        <v>0</v>
+      </c>
+      <c r="H73" t="b">
+        <v>0</v>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J73" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204176921</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J54"/>
+  <autoFilter ref="A1:J73"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 11 own-file progress (반복 12, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_11.xlsx
+++ b/output/discovery_result_11.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$73</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$74</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J73"/>
+  <dimension ref="A1:J74"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3448,8 +3448,49 @@
         </is>
       </c>
     </row>
+    <row r="74">
+      <c r="A74" t="inlineStr">
+        <is>
+          <t>1204430506</t>
+        </is>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>mongdies_jp</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>【ギフトBOX】アウアスキン ハンドクリーム＋リップバーム 2点セット フローラルモスクの香り 誕生日 出産祝い プレゼント 女性 手荒れ 唇荒れ 乾燥 敏感 高保湿ケア 手のシワ パフューム　韓国</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>モンディエス</t>
+        </is>
+      </c>
+      <c r="F74" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G74" t="n">
+        <v>0</v>
+      </c>
+      <c r="H74" t="b">
+        <v>0</v>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J74" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204430506</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J73"/>
+  <autoFilter ref="A1:J74"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 11 own-file progress (반복 15, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_11.xlsx
+++ b/output/discovery_result_11.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$74</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$83</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J74"/>
+  <dimension ref="A1:J83"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3489,8 +3489,377 @@
         </is>
       </c>
     </row>
+    <row r="75">
+      <c r="A75" t="inlineStr">
+        <is>
+          <t>1205506863</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>ohype</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>【全商品よりどり】 ボンディングケラチンフォームトリートメント200ml / ボンディングアルファケラチンヘアパック 260g / Nude Musk / Green Zest / ダメージケア</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>ohype</t>
+        </is>
+      </c>
+      <c r="F75" t="n">
+        <v>4350</v>
+      </c>
+      <c r="G75" t="n">
+        <v>1</v>
+      </c>
+      <c r="H75" t="b">
+        <v>0</v>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J75" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205506863</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>1204360681</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>ohype</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>【公式】 ボンディングアルファケラチンヘアパック 260g / Nude Musk / ジェラートヘアパック / マーブルセラピー / ダメージケア / サロンクリニック / 髪の絡まりを改善</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>ohype</t>
+        </is>
+      </c>
+      <c r="F76" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G76" t="n">
+        <v>0</v>
+      </c>
+      <c r="H76" t="b">
+        <v>0</v>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J76" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204360681</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>1203329038</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>beauty69</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>【新作】スムース＆ピュア アイス クーリング デオ スプレー 150ml 2種</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>アリウル</t>
+        </is>
+      </c>
+      <c r="F77" t="n">
+        <v>1676</v>
+      </c>
+      <c r="G77" t="n">
+        <v>0</v>
+      </c>
+      <c r="H77" t="b">
+        <v>0</v>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203329038</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>1204368140</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>CosmeticsNo1</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>ラディアンソーム100マイクロフルーダイザトナー＋エッセンス</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F78" t="n">
+        <v>21500</v>
+      </c>
+      <c r="G78" t="n">
+        <v>2</v>
+      </c>
+      <c r="H78" t="b">
+        <v>0</v>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204368140</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>1212645182</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>CosmeticsNo1</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>[1+1+1]ボルフィリン 20% アンプルスティック 10ml x 3EA</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>Derma Factory</t>
+        </is>
+      </c>
+      <c r="F79" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G79" t="n">
+        <v>0</v>
+      </c>
+      <c r="H79" t="b">
+        <v>0</v>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212645182</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>1212154060</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>CosmeticsNo1</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>[1+1+1]トラネキサム酸6%クリーム, 30ml x 3EA</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>Derma Factory</t>
+        </is>
+      </c>
+      <c r="F80" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G80" t="n">
+        <v>0</v>
+      </c>
+      <c r="H80" t="b">
+        <v>0</v>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212154060</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>1212147421</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>CosmeticsNo1</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>[1+1]トラネキサム酸6%クリーム, 30ml x 2EA</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Derma Factory</t>
+        </is>
+      </c>
+      <c r="F81" t="n">
+        <v>1750</v>
+      </c>
+      <c r="G81" t="n">
+        <v>0</v>
+      </c>
+      <c r="H81" t="b">
+        <v>0</v>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212147421</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>1199006617</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>Jurian</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>アゼライン酸16BBカーミングセラム, 30ml</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F82" t="n">
+        <v>2578</v>
+      </c>
+      <c r="G82" t="n">
+        <v>1</v>
+      </c>
+      <c r="H82" t="b">
+        <v>0</v>
+      </c>
+      <c r="I82" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199006617</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>1199701690</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>Jurian</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>カーミング バランスジェル 100ml / 水分バランス 調節</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F83" t="n">
+        <v>4735</v>
+      </c>
+      <c r="G83" t="n">
+        <v>0</v>
+      </c>
+      <c r="H83" t="b">
+        <v>0</v>
+      </c>
+      <c r="I83" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J83" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199701690</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J74"/>
+  <autoFilter ref="A1:J83"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 11 own-file progress (반복 18, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_11.xlsx
+++ b/output/discovery_result_11.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$83</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$97</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J83"/>
+  <dimension ref="A1:J97"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3858,8 +3858,582 @@
         </is>
       </c>
     </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>1171638753</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>UKB</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>ソウル 1988 セラム: レチナール リポソーム 2% + ブラックジンセン 30ml</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>K-SECRET</t>
+        </is>
+      </c>
+      <c r="F84" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G84" t="n">
+        <v>1</v>
+      </c>
+      <c r="H84" t="b">
+        <v>0</v>
+      </c>
+      <c r="I84" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171638753</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="inlineStr">
+        <is>
+          <t>1168676299</t>
+        </is>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>UKB</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>モイスチャー·レイヤ·サン·プロテクター50ml SPF50+ PA++++</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F85" t="n">
+        <v>3995</v>
+      </c>
+      <c r="G85" t="n">
+        <v>9</v>
+      </c>
+      <c r="H85" t="b">
+        <v>0</v>
+      </c>
+      <c r="I85" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168676299</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="inlineStr">
+        <is>
+          <t>1187961763</t>
+        </is>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
+          <t>heyyou</t>
+        </is>
+      </c>
+      <c r="C86" t="inlineStr">
+        <is>
+          <t>[2026] NEW 最低特典カーミング バランスジェル-保湿 / 鎮静 100ml(1+1)</t>
+        </is>
+      </c>
+      <c r="E86" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F86" t="n">
+        <v>10057</v>
+      </c>
+      <c r="G86" t="n">
+        <v>3</v>
+      </c>
+      <c r="H86" t="b">
+        <v>0</v>
+      </c>
+      <c r="I86" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1187961763</t>
+        </is>
+      </c>
+    </row>
+    <row r="87">
+      <c r="A87" t="inlineStr">
+        <is>
+          <t>1174936338</t>
+        </is>
+      </c>
+      <c r="B87" t="inlineStr">
+        <is>
+          <t>heyyou</t>
+        </is>
+      </c>
+      <c r="C87" t="inlineStr">
+        <is>
+          <t>プリジュビネーション ファーミングバクチオールセラム[童顔弾力セラム] 50ml</t>
+        </is>
+      </c>
+      <c r="E87" t="inlineStr">
+        <is>
+          <t>Dr.Jart+</t>
+        </is>
+      </c>
+      <c r="F87" t="n">
+        <v>6902</v>
+      </c>
+      <c r="G87" t="n">
+        <v>0</v>
+      </c>
+      <c r="H87" t="b">
+        <v>0</v>
+      </c>
+      <c r="I87" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174936338</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="A88" t="inlineStr">
+        <is>
+          <t>1208171928</t>
+        </is>
+      </c>
+      <c r="B88" t="inlineStr">
+        <is>
+          <t>heyyou</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
+          <t>[2026BEST] ザマトロジー 2種 セット-光彩 / 弾力(ブースター130ml+セラム45ml)</t>
+        </is>
+      </c>
+      <c r="E88" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F88" t="n">
+        <v>13046</v>
+      </c>
+      <c r="G88" t="n">
+        <v>0</v>
+      </c>
+      <c r="H88" t="b">
+        <v>0</v>
+      </c>
+      <c r="I88" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J88" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208171928</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="A89" t="inlineStr">
+        <is>
+          <t>1210644303</t>
+        </is>
+      </c>
+      <c r="B89" t="inlineStr">
+        <is>
+          <t>on_j4052</t>
+        </is>
+      </c>
+      <c r="C89" t="inlineStr">
+        <is>
+          <t>【NEW】SW19 ヘアパフュームミスト 75ml 5pm 8am 2種から選べる1種 ヘアミスト ヘアフレグランス 韓国コスメ</t>
+        </is>
+      </c>
+      <c r="E89" t="inlineStr">
+        <is>
+          <t>SW19</t>
+        </is>
+      </c>
+      <c r="F89" t="n">
+        <v>5490</v>
+      </c>
+      <c r="G89" t="n">
+        <v>0</v>
+      </c>
+      <c r="H89" t="b">
+        <v>0</v>
+      </c>
+      <c r="I89" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J89" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210644303</t>
+        </is>
+      </c>
+    </row>
+    <row r="90">
+      <c r="A90" t="inlineStr">
+        <is>
+          <t>1210988490</t>
+        </is>
+      </c>
+      <c r="B90" t="inlineStr">
+        <is>
+          <t>KBeautyMarket</t>
+        </is>
+      </c>
+      <c r="C90" t="inlineStr">
+        <is>
+          <t>[正規品] SET VQM Phytocin VIBANQM LOTION 30ml + フィニッシュローション20ml</t>
+        </is>
+      </c>
+      <c r="E90" t="inlineStr">
+        <is>
+          <t>CONAPIDIL</t>
+        </is>
+      </c>
+      <c r="F90" t="n">
+        <v>11780</v>
+      </c>
+      <c r="G90" t="n">
+        <v>0</v>
+      </c>
+      <c r="H90" t="b">
+        <v>0</v>
+      </c>
+      <c r="I90" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J90" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210988490</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="A91" t="inlineStr">
+        <is>
+          <t>1212008071</t>
+        </is>
+      </c>
+      <c r="B91" t="inlineStr">
+        <is>
+          <t>KBeautyMarket</t>
+        </is>
+      </c>
+      <c r="C91" t="inlineStr">
+        <is>
+          <t>[正規品] ナチュラル毛穴カバー乳液 韓国正規品</t>
+        </is>
+      </c>
+      <c r="E91" t="inlineStr">
+        <is>
+          <t>オブジェ</t>
+        </is>
+      </c>
+      <c r="F91" t="n">
+        <v>3070</v>
+      </c>
+      <c r="G91" t="n">
+        <v>0</v>
+      </c>
+      <c r="H91" t="b">
+        <v>0</v>
+      </c>
+      <c r="I91" t="inlineStr">
+        <is>
+          <t>120000023</t>
+        </is>
+      </c>
+      <c r="J91" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212008071</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>1211131806</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>KBeautyMarket</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>[公式販売店] ザマトロジー 2種セット[ブースター+セラム]/韓国化粧品</t>
+        </is>
+      </c>
+      <c r="E92" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F92" t="n">
+        <v>11970</v>
+      </c>
+      <c r="G92" t="n">
+        <v>1</v>
+      </c>
+      <c r="H92" t="b">
+        <v>0</v>
+      </c>
+      <c r="I92" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J92" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211131806</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>1211312549</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>KBeautyMarket</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>[公式販売店] 【1+1】 低刺激ディープクレンジング モイスチャー クレンジングオイル 145ml</t>
+        </is>
+      </c>
+      <c r="E93" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F93" t="n">
+        <v>7790</v>
+      </c>
+      <c r="G93" t="n">
+        <v>0</v>
+      </c>
+      <c r="H93" t="b">
+        <v>0</v>
+      </c>
+      <c r="I93" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J93" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211312549</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="A94" t="inlineStr">
+        <is>
+          <t>1211131359</t>
+        </is>
+      </c>
+      <c r="B94" t="inlineStr">
+        <is>
+          <t>KBeautyMarket</t>
+        </is>
+      </c>
+      <c r="C94" t="inlineStr">
+        <is>
+          <t>[公式販売店] ICD 3種 ラジアンソーム100トナー/クリーム/エッセンス</t>
+        </is>
+      </c>
+      <c r="E94" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F94" t="n">
+        <v>29990</v>
+      </c>
+      <c r="G94" t="n">
+        <v>0</v>
+      </c>
+      <c r="H94" t="b">
+        <v>0</v>
+      </c>
+      <c r="I94" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J94" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1211131359</t>
+        </is>
+      </c>
+    </row>
+    <row r="95">
+      <c r="A95" t="inlineStr">
+        <is>
+          <t>1177131836</t>
+        </is>
+      </c>
+      <c r="B95" t="inlineStr">
+        <is>
+          <t>koreahubshop</t>
+        </is>
+      </c>
+      <c r="C95" t="inlineStr">
+        <is>
+          <t>ドクターヘディソンピュア100％ビタミンCパウダー50gアンプルトナービタケア</t>
+        </is>
+      </c>
+      <c r="E95" t="inlineStr">
+        <is>
+          <t>Dr. Hedison</t>
+        </is>
+      </c>
+      <c r="F95" t="n">
+        <v>4560</v>
+      </c>
+      <c r="G95" t="n">
+        <v>0</v>
+      </c>
+      <c r="H95" t="b">
+        <v>0</v>
+      </c>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J95" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177131836</t>
+        </is>
+      </c>
+    </row>
+    <row r="96">
+      <c r="A96" t="inlineStr">
+        <is>
+          <t>1189937314</t>
+        </is>
+      </c>
+      <c r="B96" t="inlineStr">
+        <is>
+          <t>koreahubshop</t>
+        </is>
+      </c>
+      <c r="C96" t="inlineStr">
+        <is>
+          <t>アノブ ディープ ダメージ リペア シャンプー 1 + 1 ダブルセット 500ml+500ml</t>
+        </is>
+      </c>
+      <c r="E96" t="inlineStr">
+        <is>
+          <t>UNOVE</t>
+        </is>
+      </c>
+      <c r="F96" t="n">
+        <v>4840</v>
+      </c>
+      <c r="G96" t="n">
+        <v>0</v>
+      </c>
+      <c r="H96" t="b">
+        <v>0</v>
+      </c>
+      <c r="I96" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J96" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189937314</t>
+        </is>
+      </c>
+    </row>
+    <row r="97">
+      <c r="A97" t="inlineStr">
+        <is>
+          <t>1189781351</t>
+        </is>
+      </c>
+      <c r="B97" t="inlineStr">
+        <is>
+          <t>YOUSTUDIO</t>
+        </is>
+      </c>
+      <c r="C97" t="inlineStr">
+        <is>
+          <t>ブライタミン V7トーニング ライトクリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E97" t="inlineStr">
+        <is>
+          <t>Dr.Jart+</t>
+        </is>
+      </c>
+      <c r="F97" t="n">
+        <v>5299</v>
+      </c>
+      <c r="G97" t="n">
+        <v>0</v>
+      </c>
+      <c r="H97" t="b">
+        <v>0</v>
+      </c>
+      <c r="I97" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J97" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189781351</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J83"/>
+  <autoFilter ref="A1:J97"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 11 own-file progress (반복 21, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_11.xlsx
+++ b/output/discovery_result_11.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$97</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$105</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J97"/>
+  <dimension ref="A1:J105"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4432,8 +4432,336 @@
         </is>
       </c>
     </row>
+    <row r="98">
+      <c r="A98" t="inlineStr">
+        <is>
+          <t>1196020481</t>
+        </is>
+      </c>
+      <c r="B98" t="inlineStr">
+        <is>
+          <t>NDY</t>
+        </is>
+      </c>
+      <c r="C98" t="inlineStr">
+        <is>
+          <t>ツーフェイス オイルミスト 50ml 1個 基礎化粧品 保湿 潤い 艶肌 油水分バランス [並行輸入品]</t>
+        </is>
+      </c>
+      <c r="E98" t="inlineStr">
+        <is>
+          <t>インセルダーム</t>
+        </is>
+      </c>
+      <c r="F98" t="n">
+        <v>4980</v>
+      </c>
+      <c r="G98" t="n">
+        <v>2</v>
+      </c>
+      <c r="H98" t="b">
+        <v>0</v>
+      </c>
+      <c r="I98" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J98" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196020481</t>
+        </is>
+      </c>
+    </row>
+    <row r="99">
+      <c r="A99" t="inlineStr">
+        <is>
+          <t>1170033513</t>
+        </is>
+      </c>
+      <c r="B99" t="inlineStr">
+        <is>
+          <t>LuckyLucy</t>
+        </is>
+      </c>
+      <c r="C99" t="inlineStr">
+        <is>
+          <t>プレミアムペプチド ナイター 1500ショット ネックパッチ1.0,1枚 /3枚購入ごとに ペプチドトックス ボア/ 体系的管理/一日一枚の習慣で荒れていたネックラインを滑らかに~</t>
+        </is>
+      </c>
+      <c r="E99" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F99" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G99" t="n">
+        <v>0</v>
+      </c>
+      <c r="H99" t="b">
+        <v>0</v>
+      </c>
+      <c r="I99" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J99" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1170033513</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="A100" t="inlineStr">
+        <is>
+          <t>1194273240</t>
+        </is>
+      </c>
+      <c r="B100" t="inlineStr">
+        <is>
+          <t>LuckyLucy</t>
+        </is>
+      </c>
+      <c r="C100" t="inlineStr">
+        <is>
+          <t>プレミアムペプチド ナイター 1500ショット ネックパッチ1.0_1セット(4枚） /1か月集中管理/ 体系的管理/一日一枚の習慣で荒れていたネックラインを滑らかに~</t>
+        </is>
+      </c>
+      <c r="E100" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F100" t="n">
+        <v>4580</v>
+      </c>
+      <c r="G100" t="n">
+        <v>0</v>
+      </c>
+      <c r="H100" t="b">
+        <v>0</v>
+      </c>
+      <c r="I100" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J100" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194273240</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" t="inlineStr">
+        <is>
+          <t>1193753404</t>
+        </is>
+      </c>
+      <c r="B101" t="inlineStr">
+        <is>
+          <t>LuckyLucy</t>
+        </is>
+      </c>
+      <c r="C101" t="inlineStr">
+        <is>
+          <t>プレミアムペプチド ナイテ 1000 ショート ネックスティック20g+Collagen Naite Thread Neck Cream1.5ml*2ea</t>
+        </is>
+      </c>
+      <c r="E101" t="inlineStr">
+        <is>
+          <t>メディピール</t>
+        </is>
+      </c>
+      <c r="F101" t="n">
+        <v>4680</v>
+      </c>
+      <c r="G101" t="n">
+        <v>1</v>
+      </c>
+      <c r="H101" t="b">
+        <v>0</v>
+      </c>
+      <c r="I101" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J101" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193753404</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="A102" t="inlineStr">
+        <is>
+          <t>1193262729</t>
+        </is>
+      </c>
+      <c r="B102" t="inlineStr">
+        <is>
+          <t>YoiYoii</t>
+        </is>
+      </c>
+      <c r="C102" t="inlineStr">
+        <is>
+          <t>3デイズ レイヤー アンプル 55ml 美容液スキンケア,韓国スキンケア, 人気コスメ, 保湿</t>
+        </is>
+      </c>
+      <c r="E102" t="inlineStr">
+        <is>
+          <t>REVCELL</t>
+        </is>
+      </c>
+      <c r="F102" t="n">
+        <v>5848</v>
+      </c>
+      <c r="G102" t="n">
+        <v>2</v>
+      </c>
+      <c r="H102" t="b">
+        <v>0</v>
+      </c>
+      <c r="I102" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J102" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193262729</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="A103" t="inlineStr">
+        <is>
+          <t>1207093725</t>
+        </is>
+      </c>
+      <c r="B103" t="inlineStr">
+        <is>
+          <t>YoiYoii</t>
+        </is>
+      </c>
+      <c r="C103" t="inlineStr">
+        <is>
+          <t>CPR トリプルシナジーリンクルケアセラム 30ml+30ml 韓国コスメ, スキンケア,レチナール 美容液,コラーゲンセラム</t>
+        </is>
+      </c>
+      <c r="E103" t="inlineStr">
+        <is>
+          <t>THOME</t>
+        </is>
+      </c>
+      <c r="F103" t="n">
+        <v>12833</v>
+      </c>
+      <c r="G103" t="n">
+        <v>0</v>
+      </c>
+      <c r="H103" t="b">
+        <v>0</v>
+      </c>
+      <c r="I103" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J103" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1207093725</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="A104" t="inlineStr">
+        <is>
+          <t>1200649177</t>
+        </is>
+      </c>
+      <c r="B104" t="inlineStr">
+        <is>
+          <t>cosmenana</t>
+        </is>
+      </c>
+      <c r="C104" t="inlineStr">
+        <is>
+          <t>ululis ウルリス プレミアム ウォーターコンク ブラックセラム ヘアオイル 100ml 黒[3559] 宅配無料</t>
+        </is>
+      </c>
+      <c r="E104" t="inlineStr">
+        <is>
+          <t>ululis</t>
+        </is>
+      </c>
+      <c r="F104" t="n">
+        <v>1950</v>
+      </c>
+      <c r="G104" t="n">
+        <v>0</v>
+      </c>
+      <c r="H104" t="b">
+        <v>0</v>
+      </c>
+      <c r="I104" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J104" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200649177</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" t="inlineStr">
+        <is>
+          <t>1171444773</t>
+        </is>
+      </c>
+      <c r="B105" t="inlineStr">
+        <is>
+          <t>lument</t>
+        </is>
+      </c>
+      <c r="C105" t="inlineStr">
+        <is>
+          <t>【正規品 / 140ml】赤あずき クレイパック / あずきパック 毛穴 黒ずみ 角質 くすみ 洗い流す 韓国コスメ 韓国伝統成分×毛穴集中ケア</t>
+        </is>
+      </c>
+      <c r="E105" t="inlineStr">
+        <is>
+          <t>Beauty of Joseon</t>
+        </is>
+      </c>
+      <c r="F105" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G105" t="n">
+        <v>2</v>
+      </c>
+      <c r="H105" t="b">
+        <v>0</v>
+      </c>
+      <c r="I105" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J105" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171444773</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J97"/>
+  <autoFilter ref="A1:J105"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 11 own-file progress (반복 24, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_11.xlsx
+++ b/output/discovery_result_11.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$105</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$121</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J105"/>
+  <dimension ref="A1:J121"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -4760,8 +4760,664 @@
         </is>
       </c>
     </row>
+    <row r="106">
+      <c r="A106" t="inlineStr">
+        <is>
+          <t>1113959443</t>
+        </is>
+      </c>
+      <c r="B106" t="inlineStr">
+        <is>
+          <t>deos_jp</t>
+        </is>
+      </c>
+      <c r="C106" t="inlineStr">
+        <is>
+          <t>コラーゲン ロールオン アイクリーム 30ml 韓国コスメ 目元ケア ハリ ツヤ 保湿 ステンレス製3連ローラー 目元美容液</t>
+        </is>
+      </c>
+      <c r="E106" t="inlineStr">
+        <is>
+          <t>プリティースキン</t>
+        </is>
+      </c>
+      <c r="F106" t="n">
+        <v>1650</v>
+      </c>
+      <c r="G106" t="n">
+        <v>3</v>
+      </c>
+      <c r="H106" t="b">
+        <v>0</v>
+      </c>
+      <c r="I106" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J106" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1113959443</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" t="inlineStr">
+        <is>
+          <t>1179879084</t>
+        </is>
+      </c>
+      <c r="B107" t="inlineStr">
+        <is>
+          <t>deos_jp</t>
+        </is>
+      </c>
+      <c r="C107" t="inlineStr">
+        <is>
+          <t>ペプチド PDRN セラムミスト 150ml2％ローズ由来PDRN×10種ペプチドうるおいとハリを同時ケアツボクサ・セラミドNP配合乾燥対策フェイシャルミスト</t>
+        </is>
+      </c>
+      <c r="E107" t="inlineStr">
+        <is>
+          <t>プリティースキン</t>
+        </is>
+      </c>
+      <c r="F107" t="n">
+        <v>1990</v>
+      </c>
+      <c r="G107" t="n">
+        <v>0</v>
+      </c>
+      <c r="H107" t="b">
+        <v>0</v>
+      </c>
+      <c r="I107" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J107" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1179879084</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" t="inlineStr">
+        <is>
+          <t>1158581451</t>
+        </is>
+      </c>
+      <c r="B108" t="inlineStr">
+        <is>
+          <t>deos_jp</t>
+        </is>
+      </c>
+      <c r="C108" t="inlineStr">
+        <is>
+          <t>8種ヒアルロン酸 &amp;amp; ビタミン TECA クリーム (50ml) 水分爆弾 高保湿 鎮静ケア</t>
+        </is>
+      </c>
+      <c r="E108" t="inlineStr">
+        <is>
+          <t>プリティースキン</t>
+        </is>
+      </c>
+      <c r="F108" t="n">
+        <v>3270</v>
+      </c>
+      <c r="G108" t="n">
+        <v>0</v>
+      </c>
+      <c r="H108" t="b">
+        <v>0</v>
+      </c>
+      <c r="I108" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J108" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1158581451</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" t="inlineStr">
+        <is>
+          <t>1210848436</t>
+        </is>
+      </c>
+      <c r="B109" t="inlineStr">
+        <is>
+          <t>SARAHGLO</t>
+        </is>
+      </c>
+      <c r="C109" t="inlineStr">
+        <is>
+          <t>FRANZ ネイキッドスポットパッチ デュオ EARLY &amp;amp; DARK 72枚入り</t>
+        </is>
+      </c>
+      <c r="E109" t="inlineStr">
+        <is>
+          <t>FRANZ</t>
+        </is>
+      </c>
+      <c r="F109" t="n">
+        <v>3552</v>
+      </c>
+      <c r="G109" t="n">
+        <v>0</v>
+      </c>
+      <c r="H109" t="b">
+        <v>0</v>
+      </c>
+      <c r="I109" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J109" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210848436</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="A110" t="inlineStr">
+        <is>
+          <t>1157585444</t>
+        </is>
+      </c>
+      <c r="B110" t="inlineStr">
+        <is>
+          <t>JnGCommerce</t>
+        </is>
+      </c>
+      <c r="C110" t="inlineStr">
+        <is>
+          <t>トータルソリューション 24K ゴールドスネイル クレンジングフォーム 150ml</t>
+        </is>
+      </c>
+      <c r="E110" t="inlineStr">
+        <is>
+          <t>プリティースキン</t>
+        </is>
+      </c>
+      <c r="F110" t="n">
+        <v>1780</v>
+      </c>
+      <c r="G110" t="n">
+        <v>5</v>
+      </c>
+      <c r="H110" t="b">
+        <v>0</v>
+      </c>
+      <c r="I110" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J110" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1157585444</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="A111" t="inlineStr">
+        <is>
+          <t>1206727074</t>
+        </is>
+      </c>
+      <c r="B111" t="inlineStr">
+        <is>
+          <t>JnGCommerce</t>
+        </is>
+      </c>
+      <c r="C111" t="inlineStr">
+        <is>
+          <t>シカエクソソーム 保湿クリーム 60ml 鎮静 敏感肌 肌荒れケア 水分クリーム 韓国コスメ 低刺激</t>
+        </is>
+      </c>
+      <c r="E111" t="inlineStr">
+        <is>
+          <t>プリティースキン</t>
+        </is>
+      </c>
+      <c r="F111" t="n">
+        <v>2500</v>
+      </c>
+      <c r="G111" t="n">
+        <v>1</v>
+      </c>
+      <c r="H111" t="b">
+        <v>0</v>
+      </c>
+      <c r="I111" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J111" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206727074</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" t="inlineStr">
+        <is>
+          <t>1193888835</t>
+        </is>
+      </c>
+      <c r="B112" t="inlineStr">
+        <is>
+          <t>JnGCommerce</t>
+        </is>
+      </c>
+      <c r="C112" t="inlineStr">
+        <is>
+          <t>PDRN TX1 パーフェクトフィット リジュアル 幹細胞クリーム 30g/ローズ PDRN 21%配合 植物性 水分クリーム/キメケア 弾力 保湿/韓国コスメ (敏感肌/乾燥肌)/次世代スキンケア</t>
+        </is>
+      </c>
+      <c r="E112" t="inlineStr">
+        <is>
+          <t>プリティースキン</t>
+        </is>
+      </c>
+      <c r="F112" t="n">
+        <v>3990</v>
+      </c>
+      <c r="G112" t="n">
+        <v>3</v>
+      </c>
+      <c r="H112" t="b">
+        <v>0</v>
+      </c>
+      <c r="I112" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J112" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193888835</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" t="inlineStr">
+        <is>
+          <t>1180144570</t>
+        </is>
+      </c>
+      <c r="B113" t="inlineStr">
+        <is>
+          <t>yeppun</t>
+        </is>
+      </c>
+      <c r="C113" t="inlineStr">
+        <is>
+          <t>PDRN トナー250ml1個</t>
+        </is>
+      </c>
+      <c r="E113" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F113" t="n">
+        <v>3230</v>
+      </c>
+      <c r="G113" t="n">
+        <v>0</v>
+      </c>
+      <c r="H113" t="b">
+        <v>0</v>
+      </c>
+      <c r="I113" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J113" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1180144570</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" t="inlineStr">
+        <is>
+          <t>1202055978</t>
+        </is>
+      </c>
+      <c r="B114" t="inlineStr">
+        <is>
+          <t>yeppun</t>
+        </is>
+      </c>
+      <c r="C114" t="inlineStr">
+        <is>
+          <t>UVクリーム SPF50+ PA ++++ 敏感肌向けトーンアップ韓国コスメの人気日焼け止め</t>
+        </is>
+      </c>
+      <c r="E114" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F114" t="n">
+        <v>4370</v>
+      </c>
+      <c r="G114" t="n">
+        <v>0</v>
+      </c>
+      <c r="H114" t="b">
+        <v>0</v>
+      </c>
+      <c r="I114" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J114" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202055978</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="A115" t="inlineStr">
+        <is>
+          <t>1174315936</t>
+        </is>
+      </c>
+      <c r="B115" t="inlineStr">
+        <is>
+          <t>yeppun</t>
+        </is>
+      </c>
+      <c r="C115" t="inlineStr">
+        <is>
+          <t>1. マデカラボ マスク 10枚×2箱（リンクル リバイタライズ）</t>
+        </is>
+      </c>
+      <c r="E115" t="inlineStr">
+        <is>
+          <t>センテリアン24</t>
+        </is>
+      </c>
+      <c r="F115" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G115" t="n">
+        <v>0</v>
+      </c>
+      <c r="H115" t="b">
+        <v>0</v>
+      </c>
+      <c r="I115" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J115" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174315936</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="A116" t="inlineStr">
+        <is>
+          <t>1183743968</t>
+        </is>
+      </c>
+      <c r="B116" t="inlineStr">
+        <is>
+          <t>zz6o6</t>
+        </is>
+      </c>
+      <c r="C116" t="inlineStr">
+        <is>
+          <t>パーフェクト9 インテンシブ スキンケアセット 化粧水 乳液 クリーム セット スキンケア 保湿 セット 保湿</t>
+        </is>
+      </c>
+      <c r="E116" t="inlineStr">
+        <is>
+          <t>イニスフリー</t>
+        </is>
+      </c>
+      <c r="F116" t="n">
+        <v>5253</v>
+      </c>
+      <c r="G116" t="n">
+        <v>0</v>
+      </c>
+      <c r="H116" t="b">
+        <v>0</v>
+      </c>
+      <c r="I116" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J116" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183743968</t>
+        </is>
+      </c>
+    </row>
+    <row r="117">
+      <c r="A117" t="inlineStr">
+        <is>
+          <t>1177458353</t>
+        </is>
+      </c>
+      <c r="B117" t="inlineStr">
+        <is>
+          <t>zz6o6</t>
+        </is>
+      </c>
+      <c r="C117" t="inlineStr">
+        <is>
+          <t>コジサン ソープ 65g×3個 フィリピン製 ナチュラル オレンジ石鹸 ギフトにもおすすめ</t>
+        </is>
+      </c>
+      <c r="E117" t="inlineStr">
+        <is>
+          <t>こじえさん</t>
+        </is>
+      </c>
+      <c r="F117" t="n">
+        <v>2232</v>
+      </c>
+      <c r="G117" t="n">
+        <v>0</v>
+      </c>
+      <c r="H117" t="b">
+        <v>0</v>
+      </c>
+      <c r="I117" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J117" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1177458353</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="A118" t="inlineStr">
+        <is>
+          <t>1189430591</t>
+        </is>
+      </c>
+      <c r="B118" t="inlineStr">
+        <is>
+          <t>hanajini</t>
+        </is>
+      </c>
+      <c r="C118" t="inlineStr">
+        <is>
+          <t>ウォータフルトーンアップサンクリーム[ピンク], 50ml</t>
+        </is>
+      </c>
+      <c r="E118" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F118" t="n">
+        <v>2900</v>
+      </c>
+      <c r="G118" t="n">
+        <v>5</v>
+      </c>
+      <c r="H118" t="b">
+        <v>0</v>
+      </c>
+      <c r="I118" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J118" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189430591</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="A119" t="inlineStr">
+        <is>
+          <t>1198793023</t>
+        </is>
+      </c>
+      <c r="B119" t="inlineStr">
+        <is>
+          <t>hanajini</t>
+        </is>
+      </c>
+      <c r="C119" t="inlineStr">
+        <is>
+          <t>グリーンディープ ポア クレンジングバーム,100mL 1+1</t>
+        </is>
+      </c>
+      <c r="E119" t="inlineStr">
+        <is>
+          <t>ドクタージー</t>
+        </is>
+      </c>
+      <c r="F119" t="n">
+        <v>3900</v>
+      </c>
+      <c r="G119" t="n">
+        <v>7</v>
+      </c>
+      <c r="H119" t="b">
+        <v>0</v>
+      </c>
+      <c r="I119" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J119" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198793023</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="A120" t="inlineStr">
+        <is>
+          <t>1198672888</t>
+        </is>
+      </c>
+      <c r="B120" t="inlineStr">
+        <is>
+          <t>hanajini</t>
+        </is>
+      </c>
+      <c r="C120" t="inlineStr">
+        <is>
+          <t>PDRN ブースター ジェル 300mL</t>
+        </is>
+      </c>
+      <c r="E120" t="inlineStr">
+        <is>
+          <t>メディキューブ</t>
+        </is>
+      </c>
+      <c r="F120" t="n">
+        <v>2000</v>
+      </c>
+      <c r="G120" t="n">
+        <v>0</v>
+      </c>
+      <c r="H120" t="b">
+        <v>0</v>
+      </c>
+      <c r="I120" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J120" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1198672888</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="A121" t="inlineStr">
+        <is>
+          <t>1189433592</t>
+        </is>
+      </c>
+      <c r="B121" t="inlineStr">
+        <is>
+          <t>hanajini</t>
+        </is>
+      </c>
+      <c r="C121" t="inlineStr">
+        <is>
+          <t>ダブルセラム オールインワン マルチバーム 10g</t>
+        </is>
+      </c>
+      <c r="E121" t="inlineStr">
+        <is>
+          <t>ダルバ</t>
+        </is>
+      </c>
+      <c r="F121" t="n">
+        <v>3500</v>
+      </c>
+      <c r="G121" t="n">
+        <v>2</v>
+      </c>
+      <c r="H121" t="b">
+        <v>0</v>
+      </c>
+      <c r="I121" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J121" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189433592</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J105"/>
+  <autoFilter ref="A1:J121"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 11 own-file progress (반복 27, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_11.xlsx
+++ b/output/discovery_result_11.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$121</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$138</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J121"/>
+  <dimension ref="A1:J138"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5416,8 +5416,705 @@
         </is>
       </c>
     </row>
+    <row r="122">
+      <c r="A122" t="inlineStr">
+        <is>
+          <t>1209471569</t>
+        </is>
+      </c>
+      <c r="B122" t="inlineStr">
+        <is>
+          <t>khy8569</t>
+        </is>
+      </c>
+      <c r="C122" t="inlineStr">
+        <is>
+          <t>プルブア ヒノキレザー オードパルファム 30ml</t>
+        </is>
+      </c>
+      <c r="E122" t="inlineStr">
+        <is>
+          <t>pleuvoir</t>
+        </is>
+      </c>
+      <c r="F122" t="n">
+        <v>4600</v>
+      </c>
+      <c r="G122" t="n">
+        <v>0</v>
+      </c>
+      <c r="H122" t="b">
+        <v>0</v>
+      </c>
+      <c r="I122" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J122" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209471569</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="A123" t="inlineStr">
+        <is>
+          <t>1200469480</t>
+        </is>
+      </c>
+      <c r="B123" t="inlineStr">
+        <is>
+          <t>khy8569</t>
+        </is>
+      </c>
+      <c r="C123" t="inlineStr">
+        <is>
+          <t>シャドーパレット02ローズペタル데이지크 섀도우 팔레트 02로즈페탈</t>
+        </is>
+      </c>
+      <c r="E123" t="inlineStr">
+        <is>
+          <t>デイジーク</t>
+        </is>
+      </c>
+      <c r="F123" t="n">
+        <v>4200</v>
+      </c>
+      <c r="G123" t="n">
+        <v>0</v>
+      </c>
+      <c r="H123" t="b">
+        <v>0</v>
+      </c>
+      <c r="I123" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J123" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1200469480</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="A124" t="inlineStr">
+        <is>
+          <t>960305321</t>
+        </is>
+      </c>
+      <c r="B124" t="inlineStr">
+        <is>
+          <t>easymall</t>
+        </is>
+      </c>
+      <c r="C124" t="inlineStr">
+        <is>
+          <t>ボディスクラブプレステージセラピーエディション180gx4個</t>
+        </is>
+      </c>
+      <c r="E124" t="inlineStr">
+        <is>
+          <t>プル</t>
+        </is>
+      </c>
+      <c r="F124" t="n">
+        <v>4352</v>
+      </c>
+      <c r="G124" t="n">
+        <v>0</v>
+      </c>
+      <c r="H124" t="b">
+        <v>0</v>
+      </c>
+      <c r="I124" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J124" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=960305321</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="A125" t="inlineStr">
+        <is>
+          <t>960305004</t>
+        </is>
+      </c>
+      <c r="B125" t="inlineStr">
+        <is>
+          <t>easymall</t>
+        </is>
+      </c>
+      <c r="C125" t="inlineStr">
+        <is>
+          <t>ダフトアンドドフト パフュームド ボディローション エンジェルコットン 2個 300ml</t>
+        </is>
+      </c>
+      <c r="E125" t="inlineStr">
+        <is>
+          <t>ダフト&amp;amp;ドフト</t>
+        </is>
+      </c>
+      <c r="F125" t="n">
+        <v>3114</v>
+      </c>
+      <c r="G125" t="n">
+        <v>0</v>
+      </c>
+      <c r="H125" t="b">
+        <v>0</v>
+      </c>
+      <c r="I125" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J125" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=960305004</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="A126" t="inlineStr">
+        <is>
+          <t>1169665636</t>
+        </is>
+      </c>
+      <c r="B126" t="inlineStr">
+        <is>
+          <t>eightpointone</t>
+        </is>
+      </c>
+      <c r="C126" t="inlineStr">
+        <is>
+          <t>ナンバーMノーダウトコラーゲンリフティングクリーム50gホワイトニングシワ改善機能化粧品</t>
+        </is>
+      </c>
+      <c r="E126" t="inlineStr">
+        <is>
+          <t>MEDI SECTION NO.M</t>
+        </is>
+      </c>
+      <c r="F126" t="n">
+        <v>2885</v>
+      </c>
+      <c r="G126" t="n">
+        <v>1</v>
+      </c>
+      <c r="H126" t="b">
+        <v>0</v>
+      </c>
+      <c r="I126" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J126" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169665636</t>
+        </is>
+      </c>
+    </row>
+    <row r="127">
+      <c r="A127" t="inlineStr">
+        <is>
+          <t>1213011435</t>
+        </is>
+      </c>
+      <c r="B127" t="inlineStr">
+        <is>
+          <t>eightpointone</t>
+        </is>
+      </c>
+      <c r="C127" t="inlineStr">
+        <is>
+          <t>アクセンダ ルティナー 15ml スリープクリーム スリープバーム + トラベルサイズ ミニ歯磨き粉 セット</t>
+        </is>
+      </c>
+      <c r="E127" t="inlineStr">
+        <is>
+          <t>aXENDA</t>
+        </is>
+      </c>
+      <c r="F127" t="n">
+        <v>5462</v>
+      </c>
+      <c r="G127" t="n">
+        <v>0</v>
+      </c>
+      <c r="H127" t="b">
+        <v>0</v>
+      </c>
+      <c r="I127" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J127" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1213011435</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" t="inlineStr">
+        <is>
+          <t>1210202611</t>
+        </is>
+      </c>
+      <c r="B128" t="inlineStr">
+        <is>
+          <t>eightpointone</t>
+        </is>
+      </c>
+      <c r="C128" t="inlineStr">
+        <is>
+          <t>リバイブ セラピー NF アンプル / 30ml / PDRN アンプルデクスパンテノールビタミンB5</t>
+        </is>
+      </c>
+      <c r="E128" t="inlineStr">
+        <is>
+          <t>SKIN9HARI</t>
+        </is>
+      </c>
+      <c r="F128" t="n">
+        <v>3698</v>
+      </c>
+      <c r="G128" t="n">
+        <v>0</v>
+      </c>
+      <c r="H128" t="b">
+        <v>0</v>
+      </c>
+      <c r="I128" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J128" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210202611</t>
+        </is>
+      </c>
+    </row>
+    <row r="129">
+      <c r="A129" t="inlineStr">
+        <is>
+          <t>1193801185</t>
+        </is>
+      </c>
+      <c r="B129" t="inlineStr">
+        <is>
+          <t>cosmetch</t>
+        </is>
+      </c>
+      <c r="C129" t="inlineStr">
+        <is>
+          <t>【1点までメール便選択可】 レプリカ ウェン ザ レイン ストップス EDT 10ml SP (香水)</t>
+        </is>
+      </c>
+      <c r="E129" t="inlineStr">
+        <is>
+          <t>メゾンマルジェラ</t>
+        </is>
+      </c>
+      <c r="F129" t="n">
+        <v>2920</v>
+      </c>
+      <c r="G129" t="n">
+        <v>1</v>
+      </c>
+      <c r="H129" t="b">
+        <v>0</v>
+      </c>
+      <c r="I129" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J129" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1193801185</t>
+        </is>
+      </c>
+    </row>
+    <row r="130">
+      <c r="A130" t="inlineStr">
+        <is>
+          <t>1161562524</t>
+        </is>
+      </c>
+      <c r="B130" t="inlineStr">
+        <is>
+          <t>cosmetch</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
+          <t>プロディジュー フローラル オイル 100ml （全身オイル）</t>
+        </is>
+      </c>
+      <c r="E130" t="inlineStr">
+        <is>
+          <t>ニュクス</t>
+        </is>
+      </c>
+      <c r="F130" t="n">
+        <v>3110</v>
+      </c>
+      <c r="G130" t="n">
+        <v>3</v>
+      </c>
+      <c r="H130" t="b">
+        <v>0</v>
+      </c>
+      <c r="I130" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J130" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1161562524</t>
+        </is>
+      </c>
+    </row>
+    <row r="131">
+      <c r="A131" t="inlineStr">
+        <is>
+          <t>1168150897</t>
+        </is>
+      </c>
+      <c r="B131" t="inlineStr">
+        <is>
+          <t>cosmetch</t>
+        </is>
+      </c>
+      <c r="C131" t="inlineStr">
+        <is>
+          <t>ジャンヌ ランバン EDP 30ml SP （香水）</t>
+        </is>
+      </c>
+      <c r="E131" t="inlineStr">
+        <is>
+          <t>ランバン</t>
+        </is>
+      </c>
+      <c r="F131" t="n">
+        <v>2770</v>
+      </c>
+      <c r="G131" t="n">
+        <v>1</v>
+      </c>
+      <c r="H131" t="b">
+        <v>0</v>
+      </c>
+      <c r="I131" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J131" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1168150897</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="A132" t="inlineStr">
+        <is>
+          <t>1191723236</t>
+        </is>
+      </c>
+      <c r="B132" t="inlineStr">
+        <is>
+          <t>treasurebeauty</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
+          <t>ホワイトティ ジンジャーリリー ボディクリーム 400ml</t>
+        </is>
+      </c>
+      <c r="E132" t="inlineStr">
+        <is>
+          <t>エリザベスアーデン</t>
+        </is>
+      </c>
+      <c r="F132" t="n">
+        <v>3344</v>
+      </c>
+      <c r="G132" t="n">
+        <v>0</v>
+      </c>
+      <c r="H132" t="b">
+        <v>0</v>
+      </c>
+      <c r="I132" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J132" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1191723236</t>
+        </is>
+      </c>
+    </row>
+    <row r="133">
+      <c r="A133" t="inlineStr">
+        <is>
+          <t>1203745241</t>
+        </is>
+      </c>
+      <c r="B133" t="inlineStr">
+        <is>
+          <t>treasurebeauty</t>
+        </is>
+      </c>
+      <c r="C133" t="inlineStr">
+        <is>
+          <t>スキンコンディショナーエッセンシャル 330ml</t>
+        </is>
+      </c>
+      <c r="E133" t="inlineStr">
+        <is>
+          <t>アルビオン</t>
+        </is>
+      </c>
+      <c r="F133" t="n">
+        <v>10106</v>
+      </c>
+      <c r="G133" t="n">
+        <v>0</v>
+      </c>
+      <c r="H133" t="b">
+        <v>0</v>
+      </c>
+      <c r="I133" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J133" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1203745241</t>
+        </is>
+      </c>
+    </row>
+    <row r="134">
+      <c r="A134" t="inlineStr">
+        <is>
+          <t>1154890233</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>bettysbeauty</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>ロム イデアル インテンス オーデパルファン 100ml</t>
+        </is>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>ゲラン</t>
+        </is>
+      </c>
+      <c r="F134" t="n">
+        <v>20617</v>
+      </c>
+      <c r="G134" t="n">
+        <v>0</v>
+      </c>
+      <c r="H134" t="b">
+        <v>0</v>
+      </c>
+      <c r="I134" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J134" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1154890233</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
+          <t>1123998991</t>
+        </is>
+      </c>
+      <c r="B135" t="inlineStr">
+        <is>
+          <t>bettysbeauty</t>
+        </is>
+      </c>
+      <c r="C135" t="inlineStr">
+        <is>
+          <t>イリシットオーデパルファム 100ml</t>
+        </is>
+      </c>
+      <c r="E135" t="inlineStr">
+        <is>
+          <t>ジミーチュウ</t>
+        </is>
+      </c>
+      <c r="F135" t="n">
+        <v>10654</v>
+      </c>
+      <c r="G135" t="n">
+        <v>0</v>
+      </c>
+      <c r="H135" t="b">
+        <v>0</v>
+      </c>
+      <c r="I135" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J135" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1123998991</t>
+        </is>
+      </c>
+    </row>
+    <row r="136">
+      <c r="A136" t="inlineStr">
+        <is>
+          <t>1163881732</t>
+        </is>
+      </c>
+      <c r="B136" t="inlineStr">
+        <is>
+          <t>bellcosme</t>
+        </is>
+      </c>
+      <c r="C136" t="inlineStr">
+        <is>
+          <t>ロレアル セリエ ブロンディファイアー マスク 500ml</t>
+        </is>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>LOREAL PARIS</t>
+        </is>
+      </c>
+      <c r="F136" t="n">
+        <v>5374</v>
+      </c>
+      <c r="G136" t="n">
+        <v>0</v>
+      </c>
+      <c r="H136" t="b">
+        <v>0</v>
+      </c>
+      <c r="I136" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J136" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163881732</t>
+        </is>
+      </c>
+    </row>
+    <row r="137">
+      <c r="A137" t="inlineStr">
+        <is>
+          <t>1123944887</t>
+        </is>
+      </c>
+      <c r="B137" t="inlineStr">
+        <is>
+          <t>bellcosme</t>
+        </is>
+      </c>
+      <c r="C137" t="inlineStr">
+        <is>
+          <t>グリーンティー ボディローション 500ml</t>
+        </is>
+      </c>
+      <c r="E137" t="inlineStr">
+        <is>
+          <t>エリザベスアーデン</t>
+        </is>
+      </c>
+      <c r="F137" t="n">
+        <v>1679</v>
+      </c>
+      <c r="G137" t="n">
+        <v>7</v>
+      </c>
+      <c r="H137" t="b">
+        <v>0</v>
+      </c>
+      <c r="I137" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J137" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1123944887</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="A138" t="inlineStr">
+        <is>
+          <t>1204380898</t>
+        </is>
+      </c>
+      <c r="B138" t="inlineStr">
+        <is>
+          <t>bellcosme</t>
+        </is>
+      </c>
+      <c r="C138" t="inlineStr">
+        <is>
+          <t>ニューバーム ソフトムスク 40g</t>
+        </is>
+      </c>
+      <c r="E138" t="inlineStr">
+        <is>
+          <t>RETOUCH</t>
+        </is>
+      </c>
+      <c r="F138" t="n">
+        <v>2809</v>
+      </c>
+      <c r="G138" t="n">
+        <v>0</v>
+      </c>
+      <c r="H138" t="b">
+        <v>0</v>
+      </c>
+      <c r="I138" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J138" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204380898</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J121"/>
+  <autoFilter ref="A1:J138"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 11 own-file progress (반복 30, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_11.xlsx
+++ b/output/discovery_result_11.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$138</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$152</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J138"/>
+  <dimension ref="A1:J152"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -6113,8 +6113,582 @@
         </is>
       </c>
     </row>
+    <row r="139">
+      <c r="A139" t="inlineStr">
+        <is>
+          <t>1205911392</t>
+        </is>
+      </c>
+      <c r="B139" t="inlineStr">
+        <is>
+          <t>cosmetictimes</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
+          <t>ザ・モイスチャーリフト ファーミング マスク 3ml ミニサイズ</t>
+        </is>
+      </c>
+      <c r="E139" t="inlineStr">
+        <is>
+          <t>ドゥ・ラ・メール</t>
+        </is>
+      </c>
+      <c r="F139" t="n">
+        <v>2664</v>
+      </c>
+      <c r="G139" t="n">
+        <v>0</v>
+      </c>
+      <c r="H139" t="b">
+        <v>0</v>
+      </c>
+      <c r="I139" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J139" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205911392</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="A140" t="inlineStr">
+        <is>
+          <t>1205911401</t>
+        </is>
+      </c>
+      <c r="B140" t="inlineStr">
+        <is>
+          <t>cosmetictimes</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
+          <t>スキンパワー リニュー クリーム 80g</t>
+        </is>
+      </c>
+      <c r="E140" t="inlineStr">
+        <is>
+          <t>SK-Ⅱ</t>
+        </is>
+      </c>
+      <c r="F140" t="n">
+        <v>24418</v>
+      </c>
+      <c r="G140" t="n">
+        <v>0</v>
+      </c>
+      <c r="H140" t="b">
+        <v>0</v>
+      </c>
+      <c r="I140" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J140" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1205911401</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="A141" t="inlineStr">
+        <is>
+          <t>1210143801</t>
+        </is>
+      </c>
+      <c r="B141" t="inlineStr">
+        <is>
+          <t>NATSUKISHOP</t>
+        </is>
+      </c>
+      <c r="C141" t="inlineStr">
+        <is>
+          <t>DRX HQダブルブライトE　6g</t>
+        </is>
+      </c>
+      <c r="E141" t="inlineStr">
+        <is>
+          <t>ロート製薬</t>
+        </is>
+      </c>
+      <c r="F141" t="n">
+        <v>2600</v>
+      </c>
+      <c r="G141" t="n">
+        <v>0</v>
+      </c>
+      <c r="H141" t="b">
+        <v>0</v>
+      </c>
+      <c r="I141" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J141" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210143801</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="A142" t="inlineStr">
+        <is>
+          <t>1196958353</t>
+        </is>
+      </c>
+      <c r="B142" t="inlineStr">
+        <is>
+          <t>NATSUKISHOP</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
+          <t>ユーブロックスプレー 90g　2本セット　SPF50+／PA++++</t>
+        </is>
+      </c>
+      <c r="E142" t="inlineStr">
+        <is>
+          <t>サンソリット</t>
+        </is>
+      </c>
+      <c r="F142" t="n">
+        <v>3600</v>
+      </c>
+      <c r="G142" t="n">
+        <v>7</v>
+      </c>
+      <c r="H142" t="b">
+        <v>0</v>
+      </c>
+      <c r="I142" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J142" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196958353</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="A143" t="inlineStr">
+        <is>
+          <t>1189223064</t>
+        </is>
+      </c>
+      <c r="B143" t="inlineStr">
+        <is>
+          <t>tomimori</t>
+        </is>
+      </c>
+      <c r="C143" t="inlineStr">
+        <is>
+          <t>国内正規品　在庫処分　LIPOSOMEコーセー コスメデコルテ リポソームアドバンストリペアアイセラム 20mL送料無料</t>
+        </is>
+      </c>
+      <c r="E143" t="inlineStr">
+        <is>
+          <t>コスメデコルテ</t>
+        </is>
+      </c>
+      <c r="F143" t="n">
+        <v>5730</v>
+      </c>
+      <c r="G143" t="n">
+        <v>0</v>
+      </c>
+      <c r="H143" t="b">
+        <v>0</v>
+      </c>
+      <c r="I143" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J143" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1189223064</t>
+        </is>
+      </c>
+    </row>
+    <row r="144">
+      <c r="A144" t="inlineStr">
+        <is>
+          <t>1159500251</t>
+        </is>
+      </c>
+      <c r="B144" t="inlineStr">
+        <is>
+          <t>tomimori</t>
+        </is>
+      </c>
+      <c r="C144" t="inlineStr">
+        <is>
+          <t>送料無料　箱なし　shiro シロ　サボン ボディコロン 正規品</t>
+        </is>
+      </c>
+      <c r="E144" t="inlineStr">
+        <is>
+          <t>SHIRO</t>
+        </is>
+      </c>
+      <c r="F144" t="n">
+        <v>2800</v>
+      </c>
+      <c r="G144" t="n">
+        <v>0</v>
+      </c>
+      <c r="H144" t="b">
+        <v>0</v>
+      </c>
+      <c r="I144" t="inlineStr">
+        <is>
+          <t>120000022</t>
+        </is>
+      </c>
+      <c r="J144" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1159500251</t>
+        </is>
+      </c>
+    </row>
+    <row r="145">
+      <c r="A145" t="inlineStr">
+        <is>
+          <t>1210924259</t>
+        </is>
+      </c>
+      <c r="B145" t="inlineStr">
+        <is>
+          <t>tomimori</t>
+        </is>
+      </c>
+      <c r="C145" t="inlineStr">
+        <is>
+          <t>アネッサ オールインワン ビューティーパクト 1 10g SPF50+・PA+++ 日焼止め UVケア やや明るめのオークル 化粧持ち UVパクト 化粧下地 つや美肌</t>
+        </is>
+      </c>
+      <c r="E145" t="inlineStr">
+        <is>
+          <t>アネッサ</t>
+        </is>
+      </c>
+      <c r="F145" t="n">
+        <v>2980</v>
+      </c>
+      <c r="G145" t="n">
+        <v>0</v>
+      </c>
+      <c r="H145" t="b">
+        <v>0</v>
+      </c>
+      <c r="I145" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J145" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210924259</t>
+        </is>
+      </c>
+    </row>
+    <row r="146">
+      <c r="A146" t="inlineStr">
+        <is>
+          <t>1169403361</t>
+        </is>
+      </c>
+      <c r="B146" t="inlineStr">
+        <is>
+          <t>jncompany</t>
+        </is>
+      </c>
+      <c r="C146" t="inlineStr">
+        <is>
+          <t>ダーマUV365バリアハイドロミネラルサンスクリーン, [20ml*2] 40ml</t>
+        </is>
+      </c>
+      <c r="E146" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F146" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G146" t="n">
+        <v>3</v>
+      </c>
+      <c r="H146" t="b">
+        <v>0</v>
+      </c>
+      <c r="I146" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J146" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169403361</t>
+        </is>
+      </c>
+    </row>
+    <row r="147">
+      <c r="A147" t="inlineStr">
+        <is>
+          <t>1169403360</t>
+        </is>
+      </c>
+      <c r="B147" t="inlineStr">
+        <is>
+          <t>jncompany</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
+          <t>エイシカ365 水分鎮静トナー, [25ml*10] 250ml</t>
+        </is>
+      </c>
+      <c r="E147" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F147" t="n">
+        <v>1800</v>
+      </c>
+      <c r="G147" t="n">
+        <v>0</v>
+      </c>
+      <c r="H147" t="b">
+        <v>0</v>
+      </c>
+      <c r="I147" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J147" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169403360</t>
+        </is>
+      </c>
+    </row>
+    <row r="148">
+      <c r="A148" t="inlineStr">
+        <is>
+          <t>1172627984</t>
+        </is>
+      </c>
+      <c r="B148" t="inlineStr">
+        <is>
+          <t>jncompany</t>
+        </is>
+      </c>
+      <c r="C148" t="inlineStr">
+        <is>
+          <t>レチノールスーパーバウンスセラム, [10ml*3] 30ml</t>
+        </is>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>アイオペ</t>
+        </is>
+      </c>
+      <c r="F148" t="n">
+        <v>3300</v>
+      </c>
+      <c r="G148" t="n">
+        <v>6</v>
+      </c>
+      <c r="H148" t="b">
+        <v>0</v>
+      </c>
+      <c r="I148" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J148" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1172627984</t>
+        </is>
+      </c>
+    </row>
+    <row r="149">
+      <c r="A149" t="inlineStr">
+        <is>
+          <t>1169403395</t>
+        </is>
+      </c>
+      <c r="B149" t="inlineStr">
+        <is>
+          <t>jncompany</t>
+        </is>
+      </c>
+      <c r="C149" t="inlineStr">
+        <is>
+          <t>エイシカ365スージングリペアクリーム, [10ml*6] 60ml</t>
+        </is>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>AESTURA</t>
+        </is>
+      </c>
+      <c r="F149" t="n">
+        <v>2100</v>
+      </c>
+      <c r="G149" t="n">
+        <v>1</v>
+      </c>
+      <c r="H149" t="b">
+        <v>0</v>
+      </c>
+      <c r="I149" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J149" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1169403395</t>
+        </is>
+      </c>
+    </row>
+    <row r="150">
+      <c r="A150" t="inlineStr">
+        <is>
+          <t>1153736512</t>
+        </is>
+      </c>
+      <c r="B150" t="inlineStr">
+        <is>
+          <t>stellacosme</t>
+        </is>
+      </c>
+      <c r="C150" t="inlineStr">
+        <is>
+          <t>[はりんPICK] セラバリア モイスチャー アクティブトナー 200ml</t>
+        </is>
+      </c>
+      <c r="E150" t="inlineStr">
+        <is>
+          <t>ホリカホリカ</t>
+        </is>
+      </c>
+      <c r="F150" t="n">
+        <v>3601</v>
+      </c>
+      <c r="G150" t="n">
+        <v>0</v>
+      </c>
+      <c r="H150" t="b">
+        <v>0</v>
+      </c>
+      <c r="I150" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J150" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1153736512</t>
+        </is>
+      </c>
+    </row>
+    <row r="151">
+      <c r="A151" t="inlineStr">
+        <is>
+          <t>1153736555</t>
+        </is>
+      </c>
+      <c r="B151" t="inlineStr">
+        <is>
+          <t>stellacosme</t>
+        </is>
+      </c>
+      <c r="C151" t="inlineStr">
+        <is>
+          <t>[1+1] メルヘンラップ オリジナル 高周波クリーム 800ml, 2個</t>
+        </is>
+      </c>
+      <c r="E151" t="inlineStr">
+        <is>
+          <t>MARCHEN LAB</t>
+        </is>
+      </c>
+      <c r="F151" t="n">
+        <v>5530</v>
+      </c>
+      <c r="G151" t="n">
+        <v>0</v>
+      </c>
+      <c r="H151" t="b">
+        <v>0</v>
+      </c>
+      <c r="I151" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J151" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1153736555</t>
+        </is>
+      </c>
+    </row>
+    <row r="152">
+      <c r="A152" t="inlineStr">
+        <is>
+          <t>1212029919</t>
+        </is>
+      </c>
+      <c r="B152" t="inlineStr">
+        <is>
+          <t>K-CosmeMint</t>
+        </is>
+      </c>
+      <c r="C152" t="inlineStr">
+        <is>
+          <t>3番 うるツヤ発酵トナーパッド 70枚 (透明感・キメ整肌・凸凹肌卒業・肌荒れ・ 赤み鎮静・ほてりケア 毛穴引き締め ゆらぎ肌対策 角質・皮脂オフ 朝の時短・部分パック 敏感肌も安心 韓国コスメ)</t>
+        </is>
+      </c>
+      <c r="E152" t="inlineStr">
+        <is>
+          <t>ナンバーズイン</t>
+        </is>
+      </c>
+      <c r="F152" t="n">
+        <v>2150</v>
+      </c>
+      <c r="G152" t="n">
+        <v>0</v>
+      </c>
+      <c r="H152" t="b">
+        <v>0</v>
+      </c>
+      <c r="I152" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J152" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212029919</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J138"/>
+  <autoFilter ref="A1:J152"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 11 own-file progress (반복 1)
</commit_message>
<xml_diff>
--- a/output/discovery_result_11.xlsx
+++ b/output/discovery_result_11.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$315</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$328</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J315"/>
+  <dimension ref="A1:J328"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13370,8 +13370,541 @@
         </is>
       </c>
     </row>
+    <row r="316">
+      <c r="A316" t="inlineStr">
+        <is>
+          <t>1156302157</t>
+        </is>
+      </c>
+      <c r="B316" t="inlineStr">
+        <is>
+          <t>virginbeautyshop</t>
+        </is>
+      </c>
+      <c r="C316" t="inlineStr">
+        <is>
+          <t>新発売！【日本公式代理店】 ミルクバオバブ CICA ボディウォッシュ ボディローションセット サッパリ 保湿 いい匂い ボディソープ ボディーソープ 清涼</t>
+        </is>
+      </c>
+      <c r="E316" t="inlineStr">
+        <is>
+          <t>ミルクバオバブ</t>
+        </is>
+      </c>
+      <c r="F316" t="n">
+        <v>3190</v>
+      </c>
+      <c r="G316" t="n">
+        <v>1</v>
+      </c>
+      <c r="H316" t="b">
+        <v>0</v>
+      </c>
+      <c r="I316" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J316" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1156302157</t>
+        </is>
+      </c>
+    </row>
+    <row r="317">
+      <c r="A317" t="inlineStr">
+        <is>
+          <t>1054859705</t>
+        </is>
+      </c>
+      <c r="B317" t="inlineStr">
+        <is>
+          <t>calatas</t>
+        </is>
+      </c>
+      <c r="C317" t="inlineStr">
+        <is>
+          <t>【公式】サロンバイ トリートメント/350ml/選べる色【Pr/ Pk/ Nv/ Sv/Og】カラーシャンプー/ムラシャン/低刺激/保湿成分/色落ち防止/カラーキープ/美容師/サロン専売</t>
+        </is>
+      </c>
+      <c r="E317" t="inlineStr">
+        <is>
+          <t>カラタス</t>
+        </is>
+      </c>
+      <c r="F317" t="n">
+        <v>3928</v>
+      </c>
+      <c r="G317" t="n">
+        <v>3</v>
+      </c>
+      <c r="H317" t="b">
+        <v>0</v>
+      </c>
+      <c r="I317" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J317" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1054859705</t>
+        </is>
+      </c>
+    </row>
+    <row r="318">
+      <c r="A318" t="inlineStr">
+        <is>
+          <t>1185499227</t>
+        </is>
+      </c>
+      <c r="B318" t="inlineStr">
+        <is>
+          <t>shop-miyabe</t>
+        </is>
+      </c>
+      <c r="C318" t="inlineStr">
+        <is>
+          <t>エヌドット ナチュラルバーム UR 45g</t>
+        </is>
+      </c>
+      <c r="E318" t="inlineStr">
+        <is>
+          <t>ナプラ</t>
+        </is>
+      </c>
+      <c r="F318" t="n">
+        <v>1947</v>
+      </c>
+      <c r="G318" t="n">
+        <v>17</v>
+      </c>
+      <c r="H318" t="b">
+        <v>0</v>
+      </c>
+      <c r="I318" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J318" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185499227</t>
+        </is>
+      </c>
+    </row>
+    <row r="319">
+      <c r="A319" t="inlineStr">
+        <is>
+          <t>1185499226</t>
+        </is>
+      </c>
+      <c r="B319" t="inlineStr">
+        <is>
+          <t>shop-miyabe</t>
+        </is>
+      </c>
+      <c r="C319" t="inlineStr">
+        <is>
+          <t>エヌドット ポリッシュオイル UR 150ml</t>
+        </is>
+      </c>
+      <c r="E319" t="inlineStr">
+        <is>
+          <t>ナプラ</t>
+        </is>
+      </c>
+      <c r="F319" t="n">
+        <v>3289</v>
+      </c>
+      <c r="G319" t="n">
+        <v>10</v>
+      </c>
+      <c r="H319" t="b">
+        <v>0</v>
+      </c>
+      <c r="I319" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J319" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185499226</t>
+        </is>
+      </c>
+    </row>
+    <row r="320">
+      <c r="A320" t="inlineStr">
+        <is>
+          <t>1185499176</t>
+        </is>
+      </c>
+      <c r="B320" t="inlineStr">
+        <is>
+          <t>shop-miyabe</t>
+        </is>
+      </c>
+      <c r="C320" t="inlineStr">
+        <is>
+          <t>オージュアグロウシブスカルプマスク 1000g</t>
+        </is>
+      </c>
+      <c r="E320" t="inlineStr">
+        <is>
+          <t>ミルボン</t>
+        </is>
+      </c>
+      <c r="F320" t="n">
+        <v>11770</v>
+      </c>
+      <c r="G320" t="n">
+        <v>0</v>
+      </c>
+      <c r="H320" t="b">
+        <v>0</v>
+      </c>
+      <c r="I320" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J320" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185499176</t>
+        </is>
+      </c>
+    </row>
+    <row r="321">
+      <c r="A321" t="inlineStr">
+        <is>
+          <t>1141566599</t>
+        </is>
+      </c>
+      <c r="B321" t="inlineStr">
+        <is>
+          <t>k-syoten</t>
+        </is>
+      </c>
+      <c r="C321" t="inlineStr">
+        <is>
+          <t>ジングテカ トラブルセラム 50ml 75ml</t>
+        </is>
+      </c>
+      <c r="E321" t="inlineStr">
+        <is>
+          <t>bring green</t>
+        </is>
+      </c>
+      <c r="F321" t="n">
+        <v>3790</v>
+      </c>
+      <c r="G321" t="n">
+        <v>2</v>
+      </c>
+      <c r="H321" t="b">
+        <v>0</v>
+      </c>
+      <c r="I321" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J321" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1141566599</t>
+        </is>
+      </c>
+    </row>
+    <row r="322">
+      <c r="A322" t="inlineStr">
+        <is>
+          <t>1192655613</t>
+        </is>
+      </c>
+      <c r="B322" t="inlineStr">
+        <is>
+          <t>grabityofficial</t>
+        </is>
+      </c>
+      <c r="C322" t="inlineStr">
+        <is>
+          <t>【公式】 グラビティ シャンプー G0.0 Extra Strong &amp;amp; Strong 475ml</t>
+        </is>
+      </c>
+      <c r="E322" t="inlineStr">
+        <is>
+          <t>grabity</t>
+        </is>
+      </c>
+      <c r="F322" t="n">
+        <v>4500</v>
+      </c>
+      <c r="G322" t="n">
+        <v>0</v>
+      </c>
+      <c r="H322" t="b">
+        <v>0</v>
+      </c>
+      <c r="I322" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J322" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1192655613</t>
+        </is>
+      </c>
+    </row>
+    <row r="323">
+      <c r="A323" t="inlineStr">
+        <is>
+          <t>1185949288</t>
+        </is>
+      </c>
+      <c r="B323" t="inlineStr">
+        <is>
+          <t>kew82417</t>
+        </is>
+      </c>
+      <c r="C323" t="inlineStr">
+        <is>
+          <t>ラビット by ドクタージー ポアスージングクリーム 50ml</t>
+        </is>
+      </c>
+      <c r="E323" t="inlineStr">
+        <is>
+          <t>バイアウア</t>
+        </is>
+      </c>
+      <c r="F323" t="n">
+        <v>1600</v>
+      </c>
+      <c r="G323" t="n">
+        <v>0</v>
+      </c>
+      <c r="H323" t="b">
+        <v>0</v>
+      </c>
+      <c r="I323" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J323" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1185949288</t>
+        </is>
+      </c>
+    </row>
+    <row r="324">
+      <c r="A324" t="inlineStr">
+        <is>
+          <t>1201560060</t>
+        </is>
+      </c>
+      <c r="B324" t="inlineStr">
+        <is>
+          <t>danonal</t>
+        </is>
+      </c>
+      <c r="C324" t="inlineStr">
+        <is>
+          <t>ダノナル ショウブ エクソソーム スカルプセラム130ml 薬用成分配合・抜け毛ケア・頭皮鎮静</t>
+        </is>
+      </c>
+      <c r="E324" t="inlineStr">
+        <is>
+          <t>DANONAL</t>
+        </is>
+      </c>
+      <c r="F324" t="n">
+        <v>3790</v>
+      </c>
+      <c r="G324" t="n">
+        <v>0</v>
+      </c>
+      <c r="H324" t="b">
+        <v>0</v>
+      </c>
+      <c r="I324" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J324" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1201560060</t>
+        </is>
+      </c>
+    </row>
+    <row r="325">
+      <c r="A325" t="inlineStr">
+        <is>
+          <t>1209949431</t>
+        </is>
+      </c>
+      <c r="B325" t="inlineStr">
+        <is>
+          <t>droracle_official</t>
+        </is>
+      </c>
+      <c r="C325" t="inlineStr">
+        <is>
+          <t>【鎮静バリア美容液】 センテラバイオームシカアンプル 50ml CICA ゆらぎ肌 敏感肌 水分チャージ ベタつかない バリアケア 鎮静 Centella Biome</t>
+        </is>
+      </c>
+      <c r="E325" t="inlineStr">
+        <is>
+          <t>ドクターオラクル</t>
+        </is>
+      </c>
+      <c r="F325" t="n">
+        <v>4140</v>
+      </c>
+      <c r="G325" t="n">
+        <v>0</v>
+      </c>
+      <c r="H325" t="b">
+        <v>0</v>
+      </c>
+      <c r="I325" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J325" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1209949431</t>
+        </is>
+      </c>
+    </row>
+    <row r="326">
+      <c r="A326" t="inlineStr">
+        <is>
+          <t>1206813636</t>
+        </is>
+      </c>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>droracle_official</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>【鎮静サンセラム】 センテラバイオームスージングサンセラム 日焼け止め 50ml SPF50+ PA++++ CICA UVケア クーリング 紫外線ダメージ 鎮静 Centella Biome</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>ドクターオラクル</t>
+        </is>
+      </c>
+      <c r="F326" t="n">
+        <v>3680</v>
+      </c>
+      <c r="G326" t="n">
+        <v>1</v>
+      </c>
+      <c r="H326" t="b">
+        <v>0</v>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206813636</t>
+        </is>
+      </c>
+    </row>
+    <row r="327">
+      <c r="A327" t="inlineStr">
+        <is>
+          <t>1206718265</t>
+        </is>
+      </c>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>donggubat_japan</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>【NEW】【公式】 厄除けパフュームバー 豊かさの豚 パフュームバーセット / お守りプレゼント/ 韓国 香水 プレミアムディフューザー 固形石鹸 / オールインワン / GIF</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>Donggubat</t>
+        </is>
+      </c>
+      <c r="F327" t="n">
+        <v>3880</v>
+      </c>
+      <c r="G327" t="n">
+        <v>0</v>
+      </c>
+      <c r="H327" t="b">
+        <v>0</v>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206718265</t>
+        </is>
+      </c>
+    </row>
+    <row r="328">
+      <c r="A328" t="inlineStr">
+        <is>
+          <t>1202030229</t>
+        </is>
+      </c>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>donggubat_japan</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>【NEW】【公式】ダレサンアンプル 50ml / ツヤ・うるおい / メイクキープサポート・UVケア/日焼け止め/ / しっとり・ベタつきにくい/ ビタミン・ポリフェノール・ナイアシンアミ</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>Donggubat</t>
+        </is>
+      </c>
+      <c r="F328" t="n">
+        <v>4280</v>
+      </c>
+      <c r="G328" t="n">
+        <v>10</v>
+      </c>
+      <c r="H328" t="b">
+        <v>0</v>
+      </c>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202030229</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J315"/>
+  <autoFilter ref="A1:J328"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 11 own-file progress (반복 1, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_11.xlsx
+++ b/output/discovery_result_11.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$328</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$350</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J328"/>
+  <dimension ref="A1:J350"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -13903,8 +13903,910 @@
         </is>
       </c>
     </row>
+    <row r="329">
+      <c r="A329" t="inlineStr">
+        <is>
+          <t>822330209</t>
+        </is>
+      </c>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>labottach</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>AC-シオールチークニキビパッチ 4回分(8枚入) 頬にきび 肌荒れ 皮脂 集中ケア 鎮静 BHA AHA 韓国コスメ 鎮静ケア 毛穴ケア アクネ トラブル</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>Labottach</t>
+        </is>
+      </c>
+      <c r="F329" t="n">
+        <v>1000</v>
+      </c>
+      <c r="G329" t="n">
+        <v>10</v>
+      </c>
+      <c r="H329" t="b">
+        <v>0</v>
+      </c>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=822330209</t>
+        </is>
+      </c>
+    </row>
+    <row r="330">
+      <c r="A330" t="inlineStr">
+        <is>
+          <t>822324798</t>
+        </is>
+      </c>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>labottach</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>TゾーンAGフォアヘッドしわパッチ 4枚入 額のしわ 眉間のしわ しわ リフトアップ ハリ 保湿 コラーゲン ヒアルロン酸 エイジング 韓国コスメ ラボタッチ</t>
+        </is>
+      </c>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>Labottach</t>
+        </is>
+      </c>
+      <c r="F330" t="n">
+        <v>963</v>
+      </c>
+      <c r="G330" t="n">
+        <v>12</v>
+      </c>
+      <c r="H330" t="b">
+        <v>0</v>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=822324798</t>
+        </is>
+      </c>
+    </row>
+    <row r="331">
+      <c r="A331" t="inlineStr">
+        <is>
+          <t>1102160848</t>
+        </is>
+      </c>
+      <c r="B331" t="inlineStr">
+        <is>
+          <t>labottach</t>
+        </is>
+      </c>
+      <c r="C331" t="inlineStr">
+        <is>
+          <t>ダークスポットケアパッチ 32枚入 シミ そばかす 色素沈着 ニキビ跡 角層の奥へ 肌になじむ PDRN ナイアシンアミド 保湿 韓国コスメ ラボタッチ</t>
+        </is>
+      </c>
+      <c r="E331" t="inlineStr">
+        <is>
+          <t>Labottach</t>
+        </is>
+      </c>
+      <c r="F331" t="n">
+        <v>1940</v>
+      </c>
+      <c r="G331" t="n">
+        <v>4</v>
+      </c>
+      <c r="H331" t="b">
+        <v>0</v>
+      </c>
+      <c r="I331" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J331" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1102160848</t>
+        </is>
+      </c>
+    </row>
+    <row r="332">
+      <c r="A332" t="inlineStr">
+        <is>
+          <t>1162963982</t>
+        </is>
+      </c>
+      <c r="B332" t="inlineStr">
+        <is>
+          <t>lowvibe</t>
+        </is>
+      </c>
+      <c r="C332" t="inlineStr">
+        <is>
+          <t>[公式] ハンドクリーム 50ml（028 UNDRESSED / 057 WAKE UP 9 / KHAKI）</t>
+        </is>
+      </c>
+      <c r="E332" t="inlineStr">
+        <is>
+          <t>LOWVIBE</t>
+        </is>
+      </c>
+      <c r="F332" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G332" t="n">
+        <v>14</v>
+      </c>
+      <c r="H332" t="b">
+        <v>0</v>
+      </c>
+      <c r="I332" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J332" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1162963982</t>
+        </is>
+      </c>
+    </row>
+    <row r="333">
+      <c r="A333" t="inlineStr">
+        <is>
+          <t>1163067127</t>
+        </is>
+      </c>
+      <c r="B333" t="inlineStr">
+        <is>
+          <t>lowvibe</t>
+        </is>
+      </c>
+      <c r="C333" t="inlineStr">
+        <is>
+          <t>[公式] パフューム ハンドクリーム 50ml × 3本（028 UNDRESSED / 057 WAKE UP 9 / KHAKI）</t>
+        </is>
+      </c>
+      <c r="E333" t="inlineStr">
+        <is>
+          <t>LOWVIBE</t>
+        </is>
+      </c>
+      <c r="F333" t="n">
+        <v>6300</v>
+      </c>
+      <c r="G333" t="n">
+        <v>0</v>
+      </c>
+      <c r="H333" t="b">
+        <v>0</v>
+      </c>
+      <c r="I333" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J333" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1163067127</t>
+        </is>
+      </c>
+    </row>
+    <row r="334">
+      <c r="A334" t="inlineStr">
+        <is>
+          <t>1188301472</t>
+        </is>
+      </c>
+      <c r="B334" t="inlineStr">
+        <is>
+          <t>Blast_US_jp</t>
+        </is>
+      </c>
+      <c r="C334" t="inlineStr">
+        <is>
+          <t>【客室乗務員 愛用】ハンドクリーム セット 133ml×2＋75ml＋30ml 保湿・さわやかな使用感</t>
+        </is>
+      </c>
+      <c r="E334" t="inlineStr">
+        <is>
+          <t>カミール</t>
+        </is>
+      </c>
+      <c r="F334" t="n">
+        <v>2188</v>
+      </c>
+      <c r="G334" t="n">
+        <v>0</v>
+      </c>
+      <c r="H334" t="b">
+        <v>0</v>
+      </c>
+      <c r="I334" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J334" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1188301472</t>
+        </is>
+      </c>
+    </row>
+    <row r="335">
+      <c r="A335" t="inlineStr">
+        <is>
+          <t>1194211865</t>
+        </is>
+      </c>
+      <c r="B335" t="inlineStr">
+        <is>
+          <t>monclos</t>
+        </is>
+      </c>
+      <c r="C335" t="inlineStr">
+        <is>
+          <t>【公式】ケラチンボンディングヘアパックトリートメント180ml / ダメージヘア / キューティクル層保護 / ヘアケア / 根元ボリュームアップ / 静電気防止 / ハリ・コシアップ / ツヤケア</t>
+        </is>
+      </c>
+      <c r="E335" t="inlineStr">
+        <is>
+          <t>MONCLOS</t>
+        </is>
+      </c>
+      <c r="F335" t="n">
+        <v>2700</v>
+      </c>
+      <c r="G335" t="n">
+        <v>0</v>
+      </c>
+      <c r="H335" t="b">
+        <v>0</v>
+      </c>
+      <c r="I335" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J335" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194211865</t>
+        </is>
+      </c>
+    </row>
+    <row r="336">
+      <c r="A336" t="inlineStr">
+        <is>
+          <t>1183297800</t>
+        </is>
+      </c>
+      <c r="B336" t="inlineStr">
+        <is>
+          <t>monclos</t>
+        </is>
+      </c>
+      <c r="C336" t="inlineStr">
+        <is>
+          <t>【公式】コンフォート ハンドクリーム 優しい庭 30ml + キーホルダー</t>
+        </is>
+      </c>
+      <c r="E336" t="inlineStr">
+        <is>
+          <t>MONCLOS</t>
+        </is>
+      </c>
+      <c r="F336" t="n">
+        <v>2200</v>
+      </c>
+      <c r="G336" t="n">
+        <v>4</v>
+      </c>
+      <c r="H336" t="b">
+        <v>0</v>
+      </c>
+      <c r="I336" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J336" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1183297800</t>
+        </is>
+      </c>
+    </row>
+    <row r="337">
+      <c r="A337" t="inlineStr">
+        <is>
+          <t>1202024454</t>
+        </is>
+      </c>
+      <c r="B337" t="inlineStr">
+        <is>
+          <t>ichistore</t>
+        </is>
+      </c>
+      <c r="C337" t="inlineStr">
+        <is>
+          <t>常盤薬品工業 サナ なめらか本舗 豆乳イソフラボン リンクルアイクリーム N 20g 単品</t>
+        </is>
+      </c>
+      <c r="E337" t="inlineStr">
+        <is>
+          <t>なめらか本舗</t>
+        </is>
+      </c>
+      <c r="F337" t="n">
+        <v>980</v>
+      </c>
+      <c r="G337" t="n">
+        <v>3</v>
+      </c>
+      <c r="H337" t="b">
+        <v>0</v>
+      </c>
+      <c r="I337" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J337" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1202024454</t>
+        </is>
+      </c>
+    </row>
+    <row r="338">
+      <c r="A338" t="inlineStr">
+        <is>
+          <t>1176002284</t>
+        </is>
+      </c>
+      <c r="B338" t="inlineStr">
+        <is>
+          <t>ichistore</t>
+        </is>
+      </c>
+      <c r="C338" t="inlineStr">
+        <is>
+          <t>【新パッケージ】花王 アイロン用 カールローション ホワイトフローラル＆サボンの香り 110ml 単品</t>
+        </is>
+      </c>
+      <c r="E338" t="inlineStr">
+        <is>
+          <t>Liese</t>
+        </is>
+      </c>
+      <c r="F338" t="n">
+        <v>1380</v>
+      </c>
+      <c r="G338" t="n">
+        <v>3</v>
+      </c>
+      <c r="H338" t="b">
+        <v>0</v>
+      </c>
+      <c r="I338" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J338" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1176002284</t>
+        </is>
+      </c>
+    </row>
+    <row r="339">
+      <c r="A339" t="inlineStr">
+        <is>
+          <t>1208038094</t>
+        </is>
+      </c>
+      <c r="B339" t="inlineStr">
+        <is>
+          <t>ichistore</t>
+        </is>
+      </c>
+      <c r="C339" t="inlineStr">
+        <is>
+          <t>花王 ビオレ さらさらパウダーシート せっけんの香り 携帯用 10枚 × 5個 セット</t>
+        </is>
+      </c>
+      <c r="E339" t="inlineStr">
+        <is>
+          <t>ビオレ</t>
+        </is>
+      </c>
+      <c r="F339" t="n">
+        <v>1750</v>
+      </c>
+      <c r="G339" t="n">
+        <v>0</v>
+      </c>
+      <c r="H339" t="b">
+        <v>0</v>
+      </c>
+      <c r="I339" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J339" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208038094</t>
+        </is>
+      </c>
+    </row>
+    <row r="340">
+      <c r="A340" t="inlineStr">
+        <is>
+          <t>1204546255</t>
+        </is>
+      </c>
+      <c r="B340" t="inlineStr">
+        <is>
+          <t>ichistore</t>
+        </is>
+      </c>
+      <c r="C340" t="inlineStr">
+        <is>
+          <t>花王 melt メルト シャンプー クリーミーメルトフォーム 炭酸パウダー (1g x 12包) x 2個 セット</t>
+        </is>
+      </c>
+      <c r="E340" t="inlineStr">
+        <is>
+          <t>メルト</t>
+        </is>
+      </c>
+      <c r="F340" t="n">
+        <v>4180</v>
+      </c>
+      <c r="G340" t="n">
+        <v>2</v>
+      </c>
+      <c r="H340" t="b">
+        <v>0</v>
+      </c>
+      <c r="I340" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J340" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204546255</t>
+        </is>
+      </c>
+    </row>
+    <row r="341">
+      <c r="A341" t="inlineStr">
+        <is>
+          <t>1212723759</t>
+        </is>
+      </c>
+      <c r="B341" t="inlineStr">
+        <is>
+          <t>osdmarket</t>
+        </is>
+      </c>
+      <c r="C341" t="inlineStr">
+        <is>
+          <t>アクアリッチ ウォータリーエッセンス SPF50+ 120g X 2本 日焼け止め 紫外線防御効果</t>
+        </is>
+      </c>
+      <c r="E341" t="inlineStr">
+        <is>
+          <t>ビオレ</t>
+        </is>
+      </c>
+      <c r="F341" t="n">
+        <v>2300</v>
+      </c>
+      <c r="G341" t="n">
+        <v>3</v>
+      </c>
+      <c r="H341" t="b">
+        <v>0</v>
+      </c>
+      <c r="I341" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J341" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1212723759</t>
+        </is>
+      </c>
+    </row>
+    <row r="342">
+      <c r="A342" t="inlineStr">
+        <is>
+          <t>1210648122</t>
+        </is>
+      </c>
+      <c r="B342" t="inlineStr">
+        <is>
+          <t>osdmarket</t>
+        </is>
+      </c>
+      <c r="C342" t="inlineStr">
+        <is>
+          <t>ビオレu 泡ハンドソープ 詰替え用 2L 2個 大容量</t>
+        </is>
+      </c>
+      <c r="E342" t="inlineStr">
+        <is>
+          <t>ビオレ</t>
+        </is>
+      </c>
+      <c r="F342" t="n">
+        <v>3000</v>
+      </c>
+      <c r="G342" t="n">
+        <v>0</v>
+      </c>
+      <c r="H342" t="b">
+        <v>0</v>
+      </c>
+      <c r="I342" t="inlineStr">
+        <is>
+          <t>120000018</t>
+        </is>
+      </c>
+      <c r="J342" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1210648122</t>
+        </is>
+      </c>
+    </row>
+    <row r="343">
+      <c r="A343" t="inlineStr">
+        <is>
+          <t>1194053865</t>
+        </is>
+      </c>
+      <c r="B343" t="inlineStr">
+        <is>
+          <t>MOMOTOMO</t>
+        </is>
+      </c>
+      <c r="C343" t="inlineStr">
+        <is>
+          <t>【10g×4個入】 バブル スパークリング ブースター CICA / HYALON / PROGLOSS</t>
+        </is>
+      </c>
+      <c r="E343" t="inlineStr">
+        <is>
+          <t>VTコスメティックス</t>
+        </is>
+      </c>
+      <c r="F343" t="n">
+        <v>698</v>
+      </c>
+      <c r="G343" t="n">
+        <v>1</v>
+      </c>
+      <c r="H343" t="b">
+        <v>0</v>
+      </c>
+      <c r="I343" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J343" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194053865</t>
+        </is>
+      </c>
+    </row>
+    <row r="344">
+      <c r="A344" t="inlineStr">
+        <is>
+          <t>1194407001</t>
+        </is>
+      </c>
+      <c r="B344" t="inlineStr">
+        <is>
+          <t>MOMOTOMO</t>
+        </is>
+      </c>
+      <c r="C344" t="inlineStr">
+        <is>
+          <t>[1回分] 1アイバックリフト1100ショットリードルパッチ / 目元 弾力 集中ケア ニードルパッチ 改善 韓国直送</t>
+        </is>
+      </c>
+      <c r="E344" t="inlineStr">
+        <is>
+          <t>シャルド</t>
+        </is>
+      </c>
+      <c r="F344" t="n">
+        <v>1450</v>
+      </c>
+      <c r="G344" t="n">
+        <v>1</v>
+      </c>
+      <c r="H344" t="b">
+        <v>0</v>
+      </c>
+      <c r="I344" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J344" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1194407001</t>
+        </is>
+      </c>
+    </row>
+    <row r="345">
+      <c r="A345" t="inlineStr">
+        <is>
+          <t>1208281470</t>
+        </is>
+      </c>
+      <c r="B345" t="inlineStr">
+        <is>
+          <t>charde</t>
+        </is>
+      </c>
+      <c r="C345" t="inlineStr">
+        <is>
+          <t>【2026年6月新作】グルタチオン振動アイクリーム 20ml / 美顔器 / 目元ケア / くすみがちな目元ケア / トーンアップ改善</t>
+        </is>
+      </c>
+      <c r="E345" t="inlineStr">
+        <is>
+          <t>シャルド</t>
+        </is>
+      </c>
+      <c r="F345" t="n">
+        <v>3780</v>
+      </c>
+      <c r="G345" t="n">
+        <v>16</v>
+      </c>
+      <c r="H345" t="b">
+        <v>0</v>
+      </c>
+      <c r="I345" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J345" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1208281470</t>
+        </is>
+      </c>
+    </row>
+    <row r="346">
+      <c r="A346" t="inlineStr">
+        <is>
+          <t>1094120054</t>
+        </is>
+      </c>
+      <c r="B346" t="inlineStr">
+        <is>
+          <t>bihibi-jp</t>
+        </is>
+      </c>
+      <c r="C346" t="inlineStr">
+        <is>
+          <t>【日本公式代理店】韓国 アイクリーム レチノコラーゲン低分子300集中クリーム レチノール レチナール 目元たるみ 30代 40代 50代 低分子フィッシュコラーゲン しわ 目尻 ほうれい 人気</t>
+        </is>
+      </c>
+      <c r="E346" t="inlineStr">
+        <is>
+          <t>CKD_GUARANTEED</t>
+        </is>
+      </c>
+      <c r="F346" t="n">
+        <v>3800</v>
+      </c>
+      <c r="G346" t="n">
+        <v>0</v>
+      </c>
+      <c r="H346" t="b">
+        <v>0</v>
+      </c>
+      <c r="I346" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J346" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1094120054</t>
+        </is>
+      </c>
+    </row>
+    <row r="347">
+      <c r="A347" t="inlineStr">
+        <is>
+          <t>1145826907</t>
+        </is>
+      </c>
+      <c r="B347" t="inlineStr">
+        <is>
+          <t>bihibi-jp</t>
+        </is>
+      </c>
+      <c r="C347" t="inlineStr">
+        <is>
+          <t>【公式】ウォーターフィット サンセラム 日焼け止め 国内発送 シカ センテラ 韓国コスメ 水分 保湿 鎮静 低刺激 UVカット 化粧下地 紫外線</t>
+        </is>
+      </c>
+      <c r="E347" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F347" t="n">
+        <v>2530</v>
+      </c>
+      <c r="G347" t="n">
+        <v>0</v>
+      </c>
+      <c r="H347" t="b">
+        <v>0</v>
+      </c>
+      <c r="I347" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J347" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1145826907</t>
+        </is>
+      </c>
+    </row>
+    <row r="348">
+      <c r="A348" t="inlineStr">
+        <is>
+          <t>1175765151</t>
+        </is>
+      </c>
+      <c r="B348" t="inlineStr">
+        <is>
+          <t>bihibi-jp</t>
+        </is>
+      </c>
+      <c r="C348" t="inlineStr">
+        <is>
+          <t>【公式】Vita 3 ACE Aurora Toner 化粧水 保湿 ビタミン インナードライ スキンケア 韓国コスメ 水光肌 トーンアップ ニキビ跡ケア 国内発送</t>
+        </is>
+      </c>
+      <c r="E348" t="inlineStr">
+        <is>
+          <t>オーズナリー</t>
+        </is>
+      </c>
+      <c r="F348" t="n">
+        <v>2790</v>
+      </c>
+      <c r="G348" t="n">
+        <v>3</v>
+      </c>
+      <c r="H348" t="b">
+        <v>0</v>
+      </c>
+      <c r="I348" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J348" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175765151</t>
+        </is>
+      </c>
+    </row>
+    <row r="349">
+      <c r="A349" t="inlineStr">
+        <is>
+          <t>1175759418</t>
+        </is>
+      </c>
+      <c r="B349" t="inlineStr">
+        <is>
+          <t>bihibi-jp</t>
+        </is>
+      </c>
+      <c r="C349" t="inlineStr">
+        <is>
+          <t>【公式】 【LDK受賞】 Vita 3 BBC Pudding Cream ビタミン 跡ケア 保湿 高密着 スキンケア ナイトケア スリーピングパック トーンアップ</t>
+        </is>
+      </c>
+      <c r="E349" t="inlineStr">
+        <is>
+          <t>オーズナリー</t>
+        </is>
+      </c>
+      <c r="F349" t="n">
+        <v>3200</v>
+      </c>
+      <c r="G349" t="n">
+        <v>0</v>
+      </c>
+      <c r="H349" t="b">
+        <v>0</v>
+      </c>
+      <c r="I349" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J349" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1175759418</t>
+        </is>
+      </c>
+    </row>
+    <row r="350">
+      <c r="A350" t="inlineStr">
+        <is>
+          <t>1174265093</t>
+        </is>
+      </c>
+      <c r="B350" t="inlineStr">
+        <is>
+          <t>bihibi-jp</t>
+        </is>
+      </c>
+      <c r="C350" t="inlineStr">
+        <is>
+          <t>【公式】 プロバイオシカ インテンシブアンプル アンプル 50ml 美容液 鎮静 保湿 バリア ケア スキンケア センテラ ツボクサ　国内発送</t>
+        </is>
+      </c>
+      <c r="E350" t="inlineStr">
+        <is>
+          <t>SKIN1004</t>
+        </is>
+      </c>
+      <c r="F350" t="n">
+        <v>3100</v>
+      </c>
+      <c r="G350" t="n">
+        <v>4</v>
+      </c>
+      <c r="H350" t="b">
+        <v>0</v>
+      </c>
+      <c r="I350" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J350" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1174265093</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J328"/>
+  <autoFilter ref="A1:J350"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 11 own-file progress (반복 2, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_11.xlsx
+++ b/output/discovery_result_11.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$350</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$352</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J350"/>
+  <dimension ref="A1:J352"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -14805,8 +14805,90 @@
         </is>
       </c>
     </row>
+    <row r="351">
+      <c r="A351" t="inlineStr">
+        <is>
+          <t>1199108255</t>
+        </is>
+      </c>
+      <c r="B351" t="inlineStr">
+        <is>
+          <t>TROIAREUKE</t>
+        </is>
+      </c>
+      <c r="C351" t="inlineStr">
+        <is>
+          <t>【公式】【Qoo10限定セット】選べるH+ カクテルアンプル70ml＋ACSEN オイルカットクレンジング120mlの2点セット 選べる4種 肌悩み別</t>
+        </is>
+      </c>
+      <c r="E351" t="inlineStr">
+        <is>
+          <t>トロイアルケ</t>
+        </is>
+      </c>
+      <c r="F351" t="n">
+        <v>14300</v>
+      </c>
+      <c r="G351" t="n">
+        <v>17</v>
+      </c>
+      <c r="H351" t="b">
+        <v>0</v>
+      </c>
+      <c r="I351" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J351" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1199108255</t>
+        </is>
+      </c>
+    </row>
+    <row r="352">
+      <c r="A352" t="inlineStr">
+        <is>
+          <t>1164887653</t>
+        </is>
+      </c>
+      <c r="B352" t="inlineStr">
+        <is>
+          <t>TROIAREUKE</t>
+        </is>
+      </c>
+      <c r="C352" t="inlineStr">
+        <is>
+          <t>【公式】ACSEN AC スポットソリューション15ml　高濃度CICA　美容液　肌トラブルケア　肌ダメージケア　肌荒れ　赤み　ツボクサエキス</t>
+        </is>
+      </c>
+      <c r="E352" t="inlineStr">
+        <is>
+          <t>トロイアルケ</t>
+        </is>
+      </c>
+      <c r="F352" t="n">
+        <v>10560</v>
+      </c>
+      <c r="G352" t="n">
+        <v>15</v>
+      </c>
+      <c r="H352" t="b">
+        <v>0</v>
+      </c>
+      <c r="I352" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J352" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1164887653</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J350"/>
+  <autoFilter ref="A1:J352"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 11 own-file progress (반복 11, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_11.xlsx
+++ b/output/discovery_result_11.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$413</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$414</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J413"/>
+  <dimension ref="A1:J414"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17388,8 +17388,49 @@
         </is>
       </c>
     </row>
+    <row r="414">
+      <c r="A414" t="inlineStr">
+        <is>
+          <t>1171219158</t>
+        </is>
+      </c>
+      <c r="B414" t="inlineStr">
+        <is>
+          <t>aknir</t>
+        </is>
+      </c>
+      <c r="C414" t="inlineStr">
+        <is>
+          <t>AKNIR アクニー 梨花開発 薬用シャンプー トリートメント 詰め替えセット アミノ酸 頭皮ケア 保湿 くせ毛 ト ダメージ補修</t>
+        </is>
+      </c>
+      <c r="E414" t="inlineStr">
+        <is>
+          <t>AKNIR</t>
+        </is>
+      </c>
+      <c r="F414" t="n">
+        <v>9020</v>
+      </c>
+      <c r="G414" t="n">
+        <v>0</v>
+      </c>
+      <c r="H414" t="b">
+        <v>0</v>
+      </c>
+      <c r="I414" t="inlineStr">
+        <is>
+          <t>120000020</t>
+        </is>
+      </c>
+      <c r="J414" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1171219158</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J413"/>
+  <autoFilter ref="A1:J414"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Auto: parallel discovery branch 11 own-file progress (반복 4, 재시도)
</commit_message>
<xml_diff>
--- a/output/discovery_result_11.xlsx
+++ b/output/discovery_result_11.xlsx
@@ -10,7 +10,7 @@
     <sheet name="저리뷰상품" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$424</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'저리뷰상품'!$A$1:$J$428</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -429,7 +429,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J424"/>
+  <dimension ref="A1:J428"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -17839,8 +17839,172 @@
         </is>
       </c>
     </row>
+    <row r="425">
+      <c r="A425" t="inlineStr">
+        <is>
+          <t>1107189934</t>
+        </is>
+      </c>
+      <c r="B425" t="inlineStr">
+        <is>
+          <t>DEAROHNEUL</t>
+        </is>
+      </c>
+      <c r="C425" t="inlineStr">
+        <is>
+          <t>【2点セット】 DEAR OHNEUL 特許成分 DKMEX エリクサー ドンキークリーム 韓国コスメ保湿クリーム 50ml x 2 超低分子コラーゲン &amp;amp; ロバミルク 保湿/抗炎/抗酸化</t>
+        </is>
+      </c>
+      <c r="E425" t="inlineStr">
+        <is>
+          <t>Dear Ohneul</t>
+        </is>
+      </c>
+      <c r="F425" t="n">
+        <v>7700</v>
+      </c>
+      <c r="G425" t="n">
+        <v>0</v>
+      </c>
+      <c r="H425" t="b">
+        <v>0</v>
+      </c>
+      <c r="I425" t="inlineStr">
+        <is>
+          <t>120000012</t>
+        </is>
+      </c>
+      <c r="J425" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1107189934</t>
+        </is>
+      </c>
+    </row>
+    <row r="426">
+      <c r="A426" t="inlineStr">
+        <is>
+          <t>1206166293</t>
+        </is>
+      </c>
+      <c r="B426" t="inlineStr">
+        <is>
+          <t>SUMMERHOLIC</t>
+        </is>
+      </c>
+      <c r="C426" t="inlineStr">
+        <is>
+          <t>【本品+リフィル】ウルトラスポーツサンクッション15g本品+サンクッション15gリフィルUVセットSPF50+ PA++++ 日焼け止め UVケア耐水・汗対応 UVケア ヴィーガン処方</t>
+        </is>
+      </c>
+      <c r="E426" t="inlineStr">
+        <is>
+          <t>SUMMER HOLIC</t>
+        </is>
+      </c>
+      <c r="F426" t="n">
+        <v>4118</v>
+      </c>
+      <c r="G426" t="n">
+        <v>1</v>
+      </c>
+      <c r="H426" t="b">
+        <v>0</v>
+      </c>
+      <c r="I426" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J426" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1206166293</t>
+        </is>
+      </c>
+    </row>
+    <row r="427">
+      <c r="A427" t="inlineStr">
+        <is>
+          <t>1204964891</t>
+        </is>
+      </c>
+      <c r="B427" t="inlineStr">
+        <is>
+          <t>SUMMERHOLIC</t>
+        </is>
+      </c>
+      <c r="C427" t="inlineStr">
+        <is>
+          <t>【2点セット】ウルトラスポーツサンクリーム50ml＋ウルトラスポーツサンスティック19g　UVセットSPF50+ PA++++ 日焼け止め UVケア耐水・汗対応 UVケア ヴィーガン処方</t>
+        </is>
+      </c>
+      <c r="E427" t="inlineStr">
+        <is>
+          <t>SUMMER HOLIC</t>
+        </is>
+      </c>
+      <c r="F427" t="n">
+        <v>4028</v>
+      </c>
+      <c r="G427" t="n">
+        <v>3</v>
+      </c>
+      <c r="H427" t="b">
+        <v>0</v>
+      </c>
+      <c r="I427" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J427" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1204964891</t>
+        </is>
+      </c>
+    </row>
+    <row r="428">
+      <c r="A428" t="inlineStr">
+        <is>
+          <t>1196366848</t>
+        </is>
+      </c>
+      <c r="B428" t="inlineStr">
+        <is>
+          <t>SUMMERHOLIC</t>
+        </is>
+      </c>
+      <c r="C428" t="inlineStr">
+        <is>
+          <t>ウルトラスポーツサンクリーム 200ml 大容量日焼け止め</t>
+        </is>
+      </c>
+      <c r="E428" t="inlineStr">
+        <is>
+          <t>SUMMER HOLIC</t>
+        </is>
+      </c>
+      <c r="F428" t="n">
+        <v>6128</v>
+      </c>
+      <c r="G428" t="n">
+        <v>2</v>
+      </c>
+      <c r="H428" t="b">
+        <v>0</v>
+      </c>
+      <c r="I428" t="inlineStr">
+        <is>
+          <t>120000017</t>
+        </is>
+      </c>
+      <c r="J428" t="inlineStr">
+        <is>
+          <t>https://m.qoo10.jp/gmkt.inc/Mobile/Goods/goods.aspx?goodscode=1196366848</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:J424"/>
+  <autoFilter ref="A1:J428"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>